<commit_message>
Add the five Ambi stripe colourways and re-parse the library
Sam's updated filename generator adds Sage Coconut, Strawberry Merlot,
Malt Caramel, Iced Chocolate and Cloudy Sky. Regenerating naming.json
and re-parsing lifts clean names from 6,316 to 7,457 of 9,233.

Also adds --reparse so a vocabulary change no longer needs a 20-minute
re-walk, and rename-suggestions.csv listing 467 files that can be fixed
without a judgement call.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/source/Ecoy_Photography_Filename_Generator.xlsx
+++ b/assets/source/Ecoy_Photography_Filename_Generator.xlsx
@@ -14,29 +14,38 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="163">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="219" uniqueCount="173">
+  <si>
+    <t>How to use this sheet</t>
+  </si>
   <si>
     <t>Batch rename — one row per image</t>
   </si>
   <si>
+    <t>WHAT THIS IS</t>
+  </si>
+  <si>
     <t>Ecoy Photography — Filename Generator</t>
   </si>
   <si>
-    <t>How to use this sheet</t>
-  </si>
-  <si>
     <t>Product (display)</t>
   </si>
   <si>
     <t>Fill a row per photo, then copy column I into Drive as the new filename.</t>
   </si>
   <si>
+    <t>A filename generator for the Ecoy photography library. Every image is named the same way:</t>
+  </si>
+  <si>
     <t>Pick from each drop-down, then copy the green filename. Names match the live Shopify store.</t>
   </si>
   <si>
     <t>1. Product</t>
   </si>
   <si>
+    <t xml:space="preserve">      Product-Pattern-Colour-Angle-Talent/NoTalent-Real/AI-NN</t>
+  </si>
+  <si>
     <t>Product</t>
   </si>
   <si>
@@ -46,126 +55,117 @@
     <t>Colour (display)</t>
   </si>
   <si>
+    <t xml:space="preserve">      e.g.  BambooSheetSet-Solid-ForestGreen-High45-NoTalent-Real-01.jpg</t>
+  </si>
+  <si>
     <t>Colour token</t>
   </si>
   <si>
     <t>Camera angle</t>
   </si>
   <si>
-    <t>WHAT THIS IS</t>
-  </si>
-  <si>
     <t>People</t>
   </si>
   <si>
+    <t>Pattern</t>
+  </si>
+  <si>
     <t>Source</t>
   </si>
   <si>
+    <t>Colour</t>
+  </si>
+  <si>
     <t>Extension</t>
   </si>
   <si>
-    <t>Pattern</t>
+    <t>QUICK START (one file at a time)</t>
+  </si>
+  <si>
+    <t>Angle</t>
+  </si>
+  <si>
+    <t>1. Go to the 'Generator' tab.</t>
   </si>
   <si>
     <t>Pattern token</t>
   </si>
   <si>
+    <t>2. Pick each yellow drop-down.</t>
+  </si>
+  <si>
+    <t>Seq #</t>
+  </si>
+  <si>
+    <t>3. Copy the green FILENAME cell and rename the file in Google Drive.</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
     <t>Cooling Bamboo Sheet Set</t>
   </si>
   <si>
-    <t>A filename generator for the Ecoy photography library. Every image is named the same way:</t>
-  </si>
-  <si>
-    <t>Colour</t>
-  </si>
-  <si>
-    <t>Angle</t>
-  </si>
-  <si>
-    <t>Seq #</t>
-  </si>
-  <si>
-    <t>Type</t>
+    <t>DOING A WHOLE FOLDER</t>
+  </si>
+  <si>
+    <t>BambooSheetSet</t>
   </si>
   <si>
     <t>➜ FILENAME (copy)</t>
   </si>
   <si>
-    <t xml:space="preserve">      Product-Pattern-Colour-Angle-Talent/Solo-Real/AI-NN</t>
-  </si>
-  <si>
-    <t xml:space="preserve">      e.g.  BambooSheetSet-Solid-ForestGreen-High45-Solo-Real-01.jpg</t>
-  </si>
-  <si>
-    <t>BambooSheetSet</t>
+    <t>1. Go to the 'Batch' tab.  2. One row per photo.  3. Copy column I down and rename each file.</t>
   </si>
   <si>
     <t>(no colour / NA)</t>
   </si>
   <si>
-    <t>QUICK START (one file at a time)</t>
-  </si>
-  <si>
     <t>High45</t>
   </si>
   <si>
-    <t>1. Go to the 'Generator' tab.</t>
+    <t>RULES OF THUMB</t>
   </si>
   <si>
     <t>NoTalent</t>
   </si>
   <si>
-    <t>2. Pick each yellow drop-down.</t>
-  </si>
-  <si>
-    <t>3. Copy the green FILENAME cell and rename the file in Google Drive.</t>
-  </si>
-  <si>
-    <t>DOING A WHOLE FOLDER</t>
-  </si>
-  <si>
-    <t>1. Go to the 'Batch' tab.  2. One row per photo.  3. Copy column I down and rename each file.</t>
+    <t>• Product &amp; Colour names come straight from the live Shopify store (active products only).</t>
   </si>
   <si>
     <t>Real</t>
   </si>
   <si>
+    <t>• If a colour isn't in the list, it isn't live — check with Sam/Emilie before inventing one.</t>
+  </si>
+  <si>
+    <t>.jpg</t>
+  </si>
+  <si>
+    <t>(none / NA)</t>
+  </si>
+  <si>
+    <t>• Don't rename files inside the old year folders (2021-2026) — leave those alone.</t>
+  </si>
+  <si>
+    <t>Cooling Bamboo Fitted Sheet</t>
+  </si>
+  <si>
+    <t>BambooFittedSheet</t>
+  </si>
+  <si>
+    <t>Black</t>
+  </si>
+  <si>
+    <t>Low45</t>
+  </si>
+  <si>
+    <t>Talent</t>
+  </si>
+  <si>
     <t>Cooling Bamboo Quilt Cover Set</t>
   </si>
   <si>
-    <t>RULES OF THUMB</t>
-  </si>
-  <si>
-    <t>.jpg</t>
-  </si>
-  <si>
-    <t>(none / NA)</t>
-  </si>
-  <si>
-    <t>• Product &amp; Colour names come straight from the live Shopify store (active products only).</t>
-  </si>
-  <si>
-    <t>• If a colour isn't in the list, it isn't live — check with Sam/Emilie before inventing one.</t>
-  </si>
-  <si>
-    <t>Cooling Bamboo Fitted Sheet</t>
-  </si>
-  <si>
-    <t>BambooFittedSheet</t>
-  </si>
-  <si>
-    <t>• Don't rename files inside the old year folders (2021-2026) — leave those alone.</t>
-  </si>
-  <si>
-    <t>Black</t>
-  </si>
-  <si>
-    <t>Low45</t>
-  </si>
-  <si>
-    <t>Talent</t>
-  </si>
-  <si>
     <t>AI</t>
   </si>
   <si>
@@ -190,93 +190,93 @@
     <t>Overhead</t>
   </si>
   <si>
+    <t>Stripe</t>
+  </si>
+  <si>
+    <t>BambooQuiltCover</t>
+  </si>
+  <si>
+    <t>Butter</t>
+  </si>
+  <si>
     <t>2. Pattern</t>
   </si>
   <si>
-    <t>Stripe</t>
-  </si>
-  <si>
-    <t>BambooQuiltCover</t>
-  </si>
-  <si>
-    <t>Butter</t>
-  </si>
-  <si>
     <t>Freestyle</t>
   </si>
   <si>
+    <t>Polka</t>
+  </si>
+  <si>
     <t>3. Colour</t>
   </si>
   <si>
-    <t>Polka</t>
+    <t>Cooling Bamboo Pillowcase Set</t>
+  </si>
+  <si>
+    <t>BambooPillowcase</t>
   </si>
   <si>
     <t>Cookies &amp; Cream Stripe</t>
   </si>
   <si>
+    <t>Byron</t>
+  </si>
+  <si>
+    <t>CloseUp</t>
+  </si>
+  <si>
     <t>4. Camera angle</t>
   </si>
   <si>
-    <t>CloseUp</t>
-  </si>
-  <si>
-    <t>Cooling Bamboo Pillowcase Set</t>
+    <t>Bamboo European Pillowcase Set</t>
+  </si>
+  <si>
+    <t>BambooEuroPillowcase</t>
+  </si>
+  <si>
+    <t>Canyon</t>
+  </si>
+  <si>
+    <t>Deepetch</t>
   </si>
   <si>
     <t>5. People in shot?</t>
   </si>
   <si>
-    <t>BambooPillowcase</t>
-  </si>
-  <si>
-    <t>Byron</t>
-  </si>
-  <si>
-    <t>Bamboo European Pillowcase Set</t>
+    <t>Cooling Bamboo Reversible Quilt Cover (Ambi)</t>
+  </si>
+  <si>
+    <t>Matcha Forest Stripe</t>
+  </si>
+  <si>
+    <t>AmbiQuiltCover</t>
+  </si>
+  <si>
+    <t>Caramel</t>
   </si>
   <si>
     <t>6. Real photo or AI?</t>
   </si>
   <si>
-    <t>BambooEuroPillowcase</t>
-  </si>
-  <si>
-    <t>Canyon</t>
-  </si>
-  <si>
-    <t>Matcha Forest Stripe</t>
-  </si>
-  <si>
-    <t>Deepetch</t>
-  </si>
-  <si>
-    <t>Cooling Bamboo Reversible Quilt Cover (Ambi)</t>
+    <t>Side</t>
   </si>
   <si>
     <t>7. Sequence number</t>
   </si>
   <si>
-    <t>AmbiQuiltCover</t>
-  </si>
-  <si>
-    <t>Caramel</t>
-  </si>
-  <si>
-    <t>Side</t>
+    <t>Corduroy Quilt Cover Set</t>
+  </si>
+  <si>
+    <t>CordQuiltCover</t>
+  </si>
+  <si>
+    <t>Charcoal</t>
   </si>
   <si>
     <t>8. File type</t>
   </si>
   <si>
-    <t>Corduroy Quilt Cover Set</t>
-  </si>
-  <si>
-    <t>CordQuiltCover</t>
-  </si>
-  <si>
-    <t>Charcoal</t>
-  </si>
-  <si>
     <t>Flannelette Sheet Set</t>
   </si>
   <si>
@@ -463,46 +463,76 @@
     <t>MatchaForestStripe</t>
   </si>
   <si>
+    <t>Tips</t>
+  </si>
+  <si>
     <t>Burnt Peach Stripe</t>
   </si>
   <si>
     <t>BurntPeachStripe</t>
   </si>
   <si>
+    <t>• Pattern: 'Solid' = plain colour.  'Stripe' = Ambi reversible stripe.  Quilts/pillows: pick '(none / NA)'.</t>
+  </si>
+  <si>
     <t>CookiesCreamStripe</t>
   </si>
   <si>
+    <t>• 'Solo' = product only.  'Talent' = a person is in the shot.</t>
+  </si>
+  <si>
     <t>Sandy Reef Stripe</t>
   </si>
   <si>
+    <t>• 'Real' = camera photo.  'AI' = AI-generated image.</t>
+  </si>
+  <si>
     <t>SandyReefStripe</t>
   </si>
   <si>
+    <t>• Combo / 2-colour shot: file in the 'Colour A x Colour B' folder, pick the dominant colour here.</t>
+  </si>
+  <si>
     <t>Cherry Blossom Stripe</t>
   </si>
   <si>
     <t>CherryBlossomStripe</t>
   </si>
   <si>
-    <t>Tips</t>
-  </si>
-  <si>
-    <t>• Pattern: 'Solid' = plain colour.  'Stripe' = Ambi reversible stripe.  Quilts/pillows: pick '(none / NA)'.</t>
-  </si>
-  <si>
-    <t>• 'Solo' = product only.  'Talent' = a person is in the shot.</t>
-  </si>
-  <si>
-    <t>• 'Real' = camera photo.  'AI' = AI-generated image.</t>
-  </si>
-  <si>
-    <t>• Combo / 2-colour shot: file in the 'Colour A x Colour B' folder, pick the dominant colour here.</t>
-  </si>
-  <si>
     <t>• Quilts / pillows / mattress protector: choose '(no colour / NA)' for colour.</t>
   </si>
   <si>
+    <t>Iced Chocolate Stripe</t>
+  </si>
+  <si>
+    <t>IcedChocolateStripe</t>
+  </si>
+  <si>
     <t>• Renaming a whole folder? Use the 'Batch' tab.</t>
+  </si>
+  <si>
+    <t>Sage Coconut Stripe</t>
+  </si>
+  <si>
+    <t>SageCoconutStripe</t>
+  </si>
+  <si>
+    <t>Strawberry Merlot Stripe</t>
+  </si>
+  <si>
+    <t>StrawberryMerlotStripe</t>
+  </si>
+  <si>
+    <t>Malt Caramel Stripe</t>
+  </si>
+  <si>
+    <t>MaltCaramelStripe</t>
+  </si>
+  <si>
+    <t>Cloudy Sky Stripe</t>
+  </si>
+  <si>
+    <t>CloudySkyStripe</t>
   </si>
 </sst>
 </file>
@@ -523,26 +553,26 @@
       <name val="Arial"/>
     </font>
     <font>
+      <b/>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <i/>
       <sz val="10.0"/>
       <color rgb="FF555555"/>
       <name val="Arial"/>
     </font>
     <font>
-      <b/>
       <sz val="11.0"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
       <sz val="11.0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <color theme="1"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
     </font>
     <font>
@@ -558,8 +588,7 @@
     </font>
     <font>
       <color theme="1"/>
-      <name val="Calibri"/>
-      <scheme val="minor"/>
+      <name val="Arial"/>
     </font>
     <font>
       <b/>
@@ -625,7 +654,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -635,25 +664,25 @@
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="1" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="2" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
@@ -662,15 +691,19 @@
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="2" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="2" fillId="4" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="left" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
+    <xf borderId="2" fillId="4" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -907,80 +940,80 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>5</v>
+      <c r="A2" s="3" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="s">
-        <v>6</v>
+      <c r="A4" s="2" t="s">
+        <v>8</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="s">
+      <c r="A5" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>59</v>
-      </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="s">
-        <v>63</v>
+      <c r="A6" s="2" t="s">
+        <v>64</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="s">
-        <v>66</v>
+      <c r="A7" s="2" t="s">
+        <v>70</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="s">
-        <v>69</v>
+      <c r="A8" s="2" t="s">
+        <v>75</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>32</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="s">
-        <v>73</v>
+      <c r="A9" s="2" t="s">
+        <v>80</v>
       </c>
       <c r="B9" s="9" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="s">
-        <v>79</v>
+      <c r="A10" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="B10" s="9">
         <v>1.0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="s">
-        <v>83</v>
+      <c r="A11" s="2" t="s">
+        <v>86</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="s">
+      <c r="A13" s="13" t="s">
         <v>90</v>
       </c>
       <c r="B13" s="14" t="str">
@@ -989,38 +1022,38 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="s">
+      <c r="A15" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="s">
         <v>156</v>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="s">
+    <row r="19">
+      <c r="A19" s="4" t="s">
         <v>158</v>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>160</v>
-      </c>
-    </row>
     <row r="20">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="4" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="6" t="s">
-        <v>162</v>
+      <c r="A21" s="4" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1"/>
@@ -2052,69 +2085,69 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="s">
-        <v>4</v>
+      <c r="A2" s="3" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="B4" s="5" t="s">
+      <c r="A4" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F4" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G4" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H4" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I4" s="5" t="s">
-        <v>24</v>
+      <c r="F4" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="10" t="s">
-        <v>38</v>
+        <v>49</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>62</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G5" s="10">
         <v>1.0</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="I5" s="13" t="str">
+        <v>41</v>
+      </c>
+      <c r="I5" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A5,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B5,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C5,Lists!$D:$E,2,0),""),D5,E5,F5,IF(G5="","",TEXT(G5,"00")))&amp;H5</f>
         <v>BambooQuiltCover-Stripe-MatchaForestStripe-Freestyle-Talent-Real-01.jpg</v>
       </c>
@@ -2128,7 +2161,7 @@
       <c r="F6" s="10"/>
       <c r="G6" s="10"/>
       <c r="H6" s="10"/>
-      <c r="I6" s="13" t="str">
+      <c r="I6" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A6,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B6,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C6,Lists!$D:$E,2,0),""),D6,E6,F6,IF(G6="","",TEXT(G6,"00")))&amp;H6</f>
         <v/>
       </c>
@@ -2142,7 +2175,7 @@
       <c r="F7" s="10"/>
       <c r="G7" s="10"/>
       <c r="H7" s="10"/>
-      <c r="I7" s="13" t="str">
+      <c r="I7" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A7,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B7,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C7,Lists!$D:$E,2,0),""),D7,E7,F7,IF(G7="","",TEXT(G7,"00")))&amp;H7</f>
         <v/>
       </c>
@@ -2156,7 +2189,7 @@
       <c r="F8" s="10"/>
       <c r="G8" s="10"/>
       <c r="H8" s="10"/>
-      <c r="I8" s="13" t="str">
+      <c r="I8" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A8,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B8,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C8,Lists!$D:$E,2,0),""),D8,E8,F8,IF(G8="","",TEXT(G8,"00")))&amp;H8</f>
         <v/>
       </c>
@@ -2170,7 +2203,7 @@
       <c r="F9" s="10"/>
       <c r="G9" s="10"/>
       <c r="H9" s="10"/>
-      <c r="I9" s="13" t="str">
+      <c r="I9" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A9,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B9,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C9,Lists!$D:$E,2,0),""),D9,E9,F9,IF(G9="","",TEXT(G9,"00")))&amp;H9</f>
         <v/>
       </c>
@@ -2184,7 +2217,7 @@
       <c r="F10" s="10"/>
       <c r="G10" s="10"/>
       <c r="H10" s="10"/>
-      <c r="I10" s="13" t="str">
+      <c r="I10" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A10,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B10,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C10,Lists!$D:$E,2,0),""),D10,E10,F10,IF(G10="","",TEXT(G10,"00")))&amp;H10</f>
         <v/>
       </c>
@@ -2198,7 +2231,7 @@
       <c r="F11" s="10"/>
       <c r="G11" s="10"/>
       <c r="H11" s="10"/>
-      <c r="I11" s="13" t="str">
+      <c r="I11" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A11,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B11,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C11,Lists!$D:$E,2,0),""),D11,E11,F11,IF(G11="","",TEXT(G11,"00")))&amp;H11</f>
         <v/>
       </c>
@@ -2212,7 +2245,7 @@
       <c r="F12" s="10"/>
       <c r="G12" s="10"/>
       <c r="H12" s="10"/>
-      <c r="I12" s="13" t="str">
+      <c r="I12" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A12,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B12,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C12,Lists!$D:$E,2,0),""),D12,E12,F12,IF(G12="","",TEXT(G12,"00")))&amp;H12</f>
         <v/>
       </c>
@@ -2226,7 +2259,7 @@
       <c r="F13" s="10"/>
       <c r="G13" s="10"/>
       <c r="H13" s="10"/>
-      <c r="I13" s="13" t="str">
+      <c r="I13" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A13,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B13,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C13,Lists!$D:$E,2,0),""),D13,E13,F13,IF(G13="","",TEXT(G13,"00")))&amp;H13</f>
         <v/>
       </c>
@@ -2240,7 +2273,7 @@
       <c r="F14" s="10"/>
       <c r="G14" s="10"/>
       <c r="H14" s="10"/>
-      <c r="I14" s="13" t="str">
+      <c r="I14" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A14,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B14,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C14,Lists!$D:$E,2,0),""),D14,E14,F14,IF(G14="","",TEXT(G14,"00")))&amp;H14</f>
         <v/>
       </c>
@@ -2254,7 +2287,7 @@
       <c r="F15" s="10"/>
       <c r="G15" s="10"/>
       <c r="H15" s="10"/>
-      <c r="I15" s="13" t="str">
+      <c r="I15" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A15,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B15,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C15,Lists!$D:$E,2,0),""),D15,E15,F15,IF(G15="","",TEXT(G15,"00")))&amp;H15</f>
         <v/>
       </c>
@@ -2268,7 +2301,7 @@
       <c r="F16" s="10"/>
       <c r="G16" s="10"/>
       <c r="H16" s="10"/>
-      <c r="I16" s="13" t="str">
+      <c r="I16" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A16,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B16,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C16,Lists!$D:$E,2,0),""),D16,E16,F16,IF(G16="","",TEXT(G16,"00")))&amp;H16</f>
         <v/>
       </c>
@@ -2282,7 +2315,7 @@
       <c r="F17" s="10"/>
       <c r="G17" s="10"/>
       <c r="H17" s="10"/>
-      <c r="I17" s="13" t="str">
+      <c r="I17" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A17,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B17,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C17,Lists!$D:$E,2,0),""),D17,E17,F17,IF(G17="","",TEXT(G17,"00")))&amp;H17</f>
         <v/>
       </c>
@@ -2296,7 +2329,7 @@
       <c r="F18" s="10"/>
       <c r="G18" s="10"/>
       <c r="H18" s="10"/>
-      <c r="I18" s="13" t="str">
+      <c r="I18" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A18,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B18,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C18,Lists!$D:$E,2,0),""),D18,E18,F18,IF(G18="","",TEXT(G18,"00")))&amp;H18</f>
         <v/>
       </c>
@@ -2310,7 +2343,7 @@
       <c r="F19" s="10"/>
       <c r="G19" s="10"/>
       <c r="H19" s="10"/>
-      <c r="I19" s="13" t="str">
+      <c r="I19" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A19,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B19,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C19,Lists!$D:$E,2,0),""),D19,E19,F19,IF(G19="","",TEXT(G19,"00")))&amp;H19</f>
         <v/>
       </c>
@@ -2324,7 +2357,7 @@
       <c r="F20" s="10"/>
       <c r="G20" s="10"/>
       <c r="H20" s="10"/>
-      <c r="I20" s="13" t="str">
+      <c r="I20" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A20,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B20,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C20,Lists!$D:$E,2,0),""),D20,E20,F20,IF(G20="","",TEXT(G20,"00")))&amp;H20</f>
         <v/>
       </c>
@@ -2338,7 +2371,7 @@
       <c r="F21" s="10"/>
       <c r="G21" s="10"/>
       <c r="H21" s="10"/>
-      <c r="I21" s="13" t="str">
+      <c r="I21" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A21,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B21,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C21,Lists!$D:$E,2,0),""),D21,E21,F21,IF(G21="","",TEXT(G21,"00")))&amp;H21</f>
         <v/>
       </c>
@@ -2352,7 +2385,7 @@
       <c r="F22" s="10"/>
       <c r="G22" s="10"/>
       <c r="H22" s="10"/>
-      <c r="I22" s="13" t="str">
+      <c r="I22" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A22,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B22,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C22,Lists!$D:$E,2,0),""),D22,E22,F22,IF(G22="","",TEXT(G22,"00")))&amp;H22</f>
         <v/>
       </c>
@@ -2366,7 +2399,7 @@
       <c r="F23" s="10"/>
       <c r="G23" s="10"/>
       <c r="H23" s="10"/>
-      <c r="I23" s="13" t="str">
+      <c r="I23" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A23,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B23,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C23,Lists!$D:$E,2,0),""),D23,E23,F23,IF(G23="","",TEXT(G23,"00")))&amp;H23</f>
         <v/>
       </c>
@@ -2380,7 +2413,7 @@
       <c r="F24" s="10"/>
       <c r="G24" s="10"/>
       <c r="H24" s="10"/>
-      <c r="I24" s="13" t="str">
+      <c r="I24" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A24,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B24,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C24,Lists!$D:$E,2,0),""),D24,E24,F24,IF(G24="","",TEXT(G24,"00")))&amp;H24</f>
         <v/>
       </c>
@@ -2394,7 +2427,7 @@
       <c r="F25" s="10"/>
       <c r="G25" s="10"/>
       <c r="H25" s="10"/>
-      <c r="I25" s="13" t="str">
+      <c r="I25" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A25,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B25,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C25,Lists!$D:$E,2,0),""),D25,E25,F25,IF(G25="","",TEXT(G25,"00")))&amp;H25</f>
         <v/>
       </c>
@@ -2408,7 +2441,7 @@
       <c r="F26" s="10"/>
       <c r="G26" s="10"/>
       <c r="H26" s="10"/>
-      <c r="I26" s="13" t="str">
+      <c r="I26" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A26,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B26,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C26,Lists!$D:$E,2,0),""),D26,E26,F26,IF(G26="","",TEXT(G26,"00")))&amp;H26</f>
         <v/>
       </c>
@@ -2422,7 +2455,7 @@
       <c r="F27" s="10"/>
       <c r="G27" s="10"/>
       <c r="H27" s="10"/>
-      <c r="I27" s="13" t="str">
+      <c r="I27" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A27,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B27,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C27,Lists!$D:$E,2,0),""),D27,E27,F27,IF(G27="","",TEXT(G27,"00")))&amp;H27</f>
         <v/>
       </c>
@@ -2436,7 +2469,7 @@
       <c r="F28" s="10"/>
       <c r="G28" s="10"/>
       <c r="H28" s="10"/>
-      <c r="I28" s="13" t="str">
+      <c r="I28" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A28,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B28,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C28,Lists!$D:$E,2,0),""),D28,E28,F28,IF(G28="","",TEXT(G28,"00")))&amp;H28</f>
         <v/>
       </c>
@@ -2450,7 +2483,7 @@
       <c r="F29" s="10"/>
       <c r="G29" s="10"/>
       <c r="H29" s="10"/>
-      <c r="I29" s="13" t="str">
+      <c r="I29" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A29,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B29,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C29,Lists!$D:$E,2,0),""),D29,E29,F29,IF(G29="","",TEXT(G29,"00")))&amp;H29</f>
         <v/>
       </c>
@@ -2464,7 +2497,7 @@
       <c r="F30" s="10"/>
       <c r="G30" s="10"/>
       <c r="H30" s="10"/>
-      <c r="I30" s="13" t="str">
+      <c r="I30" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A30,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B30,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C30,Lists!$D:$E,2,0),""),D30,E30,F30,IF(G30="","",TEXT(G30,"00")))&amp;H30</f>
         <v/>
       </c>
@@ -2478,7 +2511,7 @@
       <c r="F31" s="10"/>
       <c r="G31" s="10"/>
       <c r="H31" s="10"/>
-      <c r="I31" s="13" t="str">
+      <c r="I31" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A31,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B31,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C31,Lists!$D:$E,2,0),""),D31,E31,F31,IF(G31="","",TEXT(G31,"00")))&amp;H31</f>
         <v/>
       </c>
@@ -2492,7 +2525,7 @@
       <c r="F32" s="10"/>
       <c r="G32" s="10"/>
       <c r="H32" s="10"/>
-      <c r="I32" s="13" t="str">
+      <c r="I32" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A32,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B32,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C32,Lists!$D:$E,2,0),""),D32,E32,F32,IF(G32="","",TEXT(G32,"00")))&amp;H32</f>
         <v/>
       </c>
@@ -2506,7 +2539,7 @@
       <c r="F33" s="10"/>
       <c r="G33" s="10"/>
       <c r="H33" s="10"/>
-      <c r="I33" s="13" t="str">
+      <c r="I33" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A33,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B33,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C33,Lists!$D:$E,2,0),""),D33,E33,F33,IF(G33="","",TEXT(G33,"00")))&amp;H33</f>
         <v/>
       </c>
@@ -2520,7 +2553,7 @@
       <c r="F34" s="10"/>
       <c r="G34" s="10"/>
       <c r="H34" s="10"/>
-      <c r="I34" s="13" t="str">
+      <c r="I34" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A34,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B34,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C34,Lists!$D:$E,2,0),""),D34,E34,F34,IF(G34="","",TEXT(G34,"00")))&amp;H34</f>
         <v/>
       </c>
@@ -2534,7 +2567,7 @@
       <c r="F35" s="10"/>
       <c r="G35" s="10"/>
       <c r="H35" s="10"/>
-      <c r="I35" s="13" t="str">
+      <c r="I35" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A35,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B35,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C35,Lists!$D:$E,2,0),""),D35,E35,F35,IF(G35="","",TEXT(G35,"00")))&amp;H35</f>
         <v/>
       </c>
@@ -2548,7 +2581,7 @@
       <c r="F36" s="10"/>
       <c r="G36" s="10"/>
       <c r="H36" s="10"/>
-      <c r="I36" s="13" t="str">
+      <c r="I36" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A36,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B36,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C36,Lists!$D:$E,2,0),""),D36,E36,F36,IF(G36="","",TEXT(G36,"00")))&amp;H36</f>
         <v/>
       </c>
@@ -2562,7 +2595,7 @@
       <c r="F37" s="10"/>
       <c r="G37" s="10"/>
       <c r="H37" s="10"/>
-      <c r="I37" s="13" t="str">
+      <c r="I37" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A37,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B37,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C37,Lists!$D:$E,2,0),""),D37,E37,F37,IF(G37="","",TEXT(G37,"00")))&amp;H37</f>
         <v/>
       </c>
@@ -2576,7 +2609,7 @@
       <c r="F38" s="10"/>
       <c r="G38" s="10"/>
       <c r="H38" s="10"/>
-      <c r="I38" s="13" t="str">
+      <c r="I38" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A38,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B38,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C38,Lists!$D:$E,2,0),""),D38,E38,F38,IF(G38="","",TEXT(G38,"00")))&amp;H38</f>
         <v/>
       </c>
@@ -2590,7 +2623,7 @@
       <c r="F39" s="10"/>
       <c r="G39" s="10"/>
       <c r="H39" s="10"/>
-      <c r="I39" s="13" t="str">
+      <c r="I39" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A39,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B39,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C39,Lists!$D:$E,2,0),""),D39,E39,F39,IF(G39="","",TEXT(G39,"00")))&amp;H39</f>
         <v/>
       </c>
@@ -2604,7 +2637,7 @@
       <c r="F40" s="10"/>
       <c r="G40" s="10"/>
       <c r="H40" s="10"/>
-      <c r="I40" s="13" t="str">
+      <c r="I40" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A40,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B40,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C40,Lists!$D:$E,2,0),""),D40,E40,F40,IF(G40="","",TEXT(G40,"00")))&amp;H40</f>
         <v/>
       </c>
@@ -2618,7 +2651,7 @@
       <c r="F41" s="10"/>
       <c r="G41" s="10"/>
       <c r="H41" s="10"/>
-      <c r="I41" s="13" t="str">
+      <c r="I41" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A41,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B41,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C41,Lists!$D:$E,2,0),""),D41,E41,F41,IF(G41="","",TEXT(G41,"00")))&amp;H41</f>
         <v/>
       </c>
@@ -2632,7 +2665,7 @@
       <c r="F42" s="10"/>
       <c r="G42" s="10"/>
       <c r="H42" s="10"/>
-      <c r="I42" s="13" t="str">
+      <c r="I42" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A42,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B42,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C42,Lists!$D:$E,2,0),""),D42,E42,F42,IF(G42="","",TEXT(G42,"00")))&amp;H42</f>
         <v/>
       </c>
@@ -2646,7 +2679,7 @@
       <c r="F43" s="10"/>
       <c r="G43" s="10"/>
       <c r="H43" s="10"/>
-      <c r="I43" s="13" t="str">
+      <c r="I43" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A43,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B43,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C43,Lists!$D:$E,2,0),""),D43,E43,F43,IF(G43="","",TEXT(G43,"00")))&amp;H43</f>
         <v/>
       </c>
@@ -2660,7 +2693,7 @@
       <c r="F44" s="10"/>
       <c r="G44" s="10"/>
       <c r="H44" s="10"/>
-      <c r="I44" s="13" t="str">
+      <c r="I44" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A44,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B44,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C44,Lists!$D:$E,2,0),""),D44,E44,F44,IF(G44="","",TEXT(G44,"00")))&amp;H44</f>
         <v/>
       </c>
@@ -2674,7 +2707,7 @@
       <c r="F45" s="10"/>
       <c r="G45" s="10"/>
       <c r="H45" s="10"/>
-      <c r="I45" s="13" t="str">
+      <c r="I45" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A45,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B45,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C45,Lists!$D:$E,2,0),""),D45,E45,F45,IF(G45="","",TEXT(G45,"00")))&amp;H45</f>
         <v/>
       </c>
@@ -2688,7 +2721,7 @@
       <c r="F46" s="10"/>
       <c r="G46" s="10"/>
       <c r="H46" s="10"/>
-      <c r="I46" s="13" t="str">
+      <c r="I46" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A46,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B46,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C46,Lists!$D:$E,2,0),""),D46,E46,F46,IF(G46="","",TEXT(G46,"00")))&amp;H46</f>
         <v/>
       </c>
@@ -2702,7 +2735,7 @@
       <c r="F47" s="10"/>
       <c r="G47" s="10"/>
       <c r="H47" s="10"/>
-      <c r="I47" s="13" t="str">
+      <c r="I47" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A47,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B47,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C47,Lists!$D:$E,2,0),""),D47,E47,F47,IF(G47="","",TEXT(G47,"00")))&amp;H47</f>
         <v/>
       </c>
@@ -2716,7 +2749,7 @@
       <c r="F48" s="10"/>
       <c r="G48" s="10"/>
       <c r="H48" s="10"/>
-      <c r="I48" s="13" t="str">
+      <c r="I48" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A48,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B48,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C48,Lists!$D:$E,2,0),""),D48,E48,F48,IF(G48="","",TEXT(G48,"00")))&amp;H48</f>
         <v/>
       </c>
@@ -2730,7 +2763,7 @@
       <c r="F49" s="10"/>
       <c r="G49" s="10"/>
       <c r="H49" s="10"/>
-      <c r="I49" s="13" t="str">
+      <c r="I49" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A49,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B49,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C49,Lists!$D:$E,2,0),""),D49,E49,F49,IF(G49="","",TEXT(G49,"00")))&amp;H49</f>
         <v/>
       </c>
@@ -2744,7 +2777,7 @@
       <c r="F50" s="10"/>
       <c r="G50" s="10"/>
       <c r="H50" s="10"/>
-      <c r="I50" s="13" t="str">
+      <c r="I50" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A50,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B50,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C50,Lists!$D:$E,2,0),""),D50,E50,F50,IF(G50="","",TEXT(G50,"00")))&amp;H50</f>
         <v/>
       </c>
@@ -2758,7 +2791,7 @@
       <c r="F51" s="10"/>
       <c r="G51" s="10"/>
       <c r="H51" s="10"/>
-      <c r="I51" s="13" t="str">
+      <c r="I51" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A51,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B51,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C51,Lists!$D:$E,2,0),""),D51,E51,F51,IF(G51="","",TEXT(G51,"00")))&amp;H51</f>
         <v/>
       </c>
@@ -2772,7 +2805,7 @@
       <c r="F52" s="10"/>
       <c r="G52" s="10"/>
       <c r="H52" s="10"/>
-      <c r="I52" s="13" t="str">
+      <c r="I52" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A52,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B52,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C52,Lists!$D:$E,2,0),""),D52,E52,F52,IF(G52="","",TEXT(G52,"00")))&amp;H52</f>
         <v/>
       </c>
@@ -2786,7 +2819,7 @@
       <c r="F53" s="10"/>
       <c r="G53" s="10"/>
       <c r="H53" s="10"/>
-      <c r="I53" s="13" t="str">
+      <c r="I53" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A53,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B53,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C53,Lists!$D:$E,2,0),""),D53,E53,F53,IF(G53="","",TEXT(G53,"00")))&amp;H53</f>
         <v/>
       </c>
@@ -2800,7 +2833,7 @@
       <c r="F54" s="10"/>
       <c r="G54" s="10"/>
       <c r="H54" s="10"/>
-      <c r="I54" s="13" t="str">
+      <c r="I54" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A54,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B54,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C54,Lists!$D:$E,2,0),""),D54,E54,F54,IF(G54="","",TEXT(G54,"00")))&amp;H54</f>
         <v/>
       </c>
@@ -2814,7 +2847,7 @@
       <c r="F55" s="10"/>
       <c r="G55" s="10"/>
       <c r="H55" s="10"/>
-      <c r="I55" s="13" t="str">
+      <c r="I55" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A55,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B55,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C55,Lists!$D:$E,2,0),""),D55,E55,F55,IF(G55="","",TEXT(G55,"00")))&amp;H55</f>
         <v/>
       </c>
@@ -2828,7 +2861,7 @@
       <c r="F56" s="10"/>
       <c r="G56" s="10"/>
       <c r="H56" s="10"/>
-      <c r="I56" s="13" t="str">
+      <c r="I56" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A56,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B56,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C56,Lists!$D:$E,2,0),""),D56,E56,F56,IF(G56="","",TEXT(G56,"00")))&amp;H56</f>
         <v/>
       </c>
@@ -2842,7 +2875,7 @@
       <c r="F57" s="10"/>
       <c r="G57" s="10"/>
       <c r="H57" s="10"/>
-      <c r="I57" s="13" t="str">
+      <c r="I57" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A57,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B57,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C57,Lists!$D:$E,2,0),""),D57,E57,F57,IF(G57="","",TEXT(G57,"00")))&amp;H57</f>
         <v/>
       </c>
@@ -2856,7 +2889,7 @@
       <c r="F58" s="10"/>
       <c r="G58" s="10"/>
       <c r="H58" s="10"/>
-      <c r="I58" s="13" t="str">
+      <c r="I58" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A58,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B58,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C58,Lists!$D:$E,2,0),""),D58,E58,F58,IF(G58="","",TEXT(G58,"00")))&amp;H58</f>
         <v/>
       </c>
@@ -2870,7 +2903,7 @@
       <c r="F59" s="10"/>
       <c r="G59" s="10"/>
       <c r="H59" s="10"/>
-      <c r="I59" s="13" t="str">
+      <c r="I59" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A59,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B59,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C59,Lists!$D:$E,2,0),""),D59,E59,F59,IF(G59="","",TEXT(G59,"00")))&amp;H59</f>
         <v/>
       </c>
@@ -2884,7 +2917,7 @@
       <c r="F60" s="10"/>
       <c r="G60" s="10"/>
       <c r="H60" s="10"/>
-      <c r="I60" s="13" t="str">
+      <c r="I60" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A60,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B60,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C60,Lists!$D:$E,2,0),""),D60,E60,F60,IF(G60="","",TEXT(G60,"00")))&amp;H60</f>
         <v/>
       </c>
@@ -2898,7 +2931,7 @@
       <c r="F61" s="10"/>
       <c r="G61" s="10"/>
       <c r="H61" s="10"/>
-      <c r="I61" s="13" t="str">
+      <c r="I61" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A61,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B61,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C61,Lists!$D:$E,2,0),""),D61,E61,F61,IF(G61="","",TEXT(G61,"00")))&amp;H61</f>
         <v/>
       </c>
@@ -2912,7 +2945,7 @@
       <c r="F62" s="10"/>
       <c r="G62" s="10"/>
       <c r="H62" s="10"/>
-      <c r="I62" s="13" t="str">
+      <c r="I62" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A62,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B62,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C62,Lists!$D:$E,2,0),""),D62,E62,F62,IF(G62="","",TEXT(G62,"00")))&amp;H62</f>
         <v/>
       </c>
@@ -2926,7 +2959,7 @@
       <c r="F63" s="10"/>
       <c r="G63" s="10"/>
       <c r="H63" s="10"/>
-      <c r="I63" s="13" t="str">
+      <c r="I63" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A63,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B63,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C63,Lists!$D:$E,2,0),""),D63,E63,F63,IF(G63="","",TEXT(G63,"00")))&amp;H63</f>
         <v/>
       </c>
@@ -2940,7 +2973,7 @@
       <c r="F64" s="10"/>
       <c r="G64" s="10"/>
       <c r="H64" s="10"/>
-      <c r="I64" s="13" t="str">
+      <c r="I64" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A64,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B64,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C64,Lists!$D:$E,2,0),""),D64,E64,F64,IF(G64="","",TEXT(G64,"00")))&amp;H64</f>
         <v/>
       </c>
@@ -2954,7 +2987,7 @@
       <c r="F65" s="10"/>
       <c r="G65" s="10"/>
       <c r="H65" s="10"/>
-      <c r="I65" s="13" t="str">
+      <c r="I65" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A65,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B65,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C65,Lists!$D:$E,2,0),""),D65,E65,F65,IF(G65="","",TEXT(G65,"00")))&amp;H65</f>
         <v/>
       </c>
@@ -2968,7 +3001,7 @@
       <c r="F66" s="10"/>
       <c r="G66" s="10"/>
       <c r="H66" s="10"/>
-      <c r="I66" s="13" t="str">
+      <c r="I66" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A66,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B66,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C66,Lists!$D:$E,2,0),""),D66,E66,F66,IF(G66="","",TEXT(G66,"00")))&amp;H66</f>
         <v/>
       </c>
@@ -2982,7 +3015,7 @@
       <c r="F67" s="10"/>
       <c r="G67" s="10"/>
       <c r="H67" s="10"/>
-      <c r="I67" s="13" t="str">
+      <c r="I67" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A67,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B67,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C67,Lists!$D:$E,2,0),""),D67,E67,F67,IF(G67="","",TEXT(G67,"00")))&amp;H67</f>
         <v/>
       </c>
@@ -2996,7 +3029,7 @@
       <c r="F68" s="10"/>
       <c r="G68" s="10"/>
       <c r="H68" s="10"/>
-      <c r="I68" s="13" t="str">
+      <c r="I68" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A68,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B68,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C68,Lists!$D:$E,2,0),""),D68,E68,F68,IF(G68="","",TEXT(G68,"00")))&amp;H68</f>
         <v/>
       </c>
@@ -3010,7 +3043,7 @@
       <c r="F69" s="10"/>
       <c r="G69" s="10"/>
       <c r="H69" s="10"/>
-      <c r="I69" s="13" t="str">
+      <c r="I69" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A69,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B69,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C69,Lists!$D:$E,2,0),""),D69,E69,F69,IF(G69="","",TEXT(G69,"00")))&amp;H69</f>
         <v/>
       </c>
@@ -3024,7 +3057,7 @@
       <c r="F70" s="10"/>
       <c r="G70" s="10"/>
       <c r="H70" s="10"/>
-      <c r="I70" s="13" t="str">
+      <c r="I70" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A70,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B70,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C70,Lists!$D:$E,2,0),""),D70,E70,F70,IF(G70="","",TEXT(G70,"00")))&amp;H70</f>
         <v/>
       </c>
@@ -3038,7 +3071,7 @@
       <c r="F71" s="10"/>
       <c r="G71" s="10"/>
       <c r="H71" s="10"/>
-      <c r="I71" s="13" t="str">
+      <c r="I71" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A71,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B71,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C71,Lists!$D:$E,2,0),""),D71,E71,F71,IF(G71="","",TEXT(G71,"00")))&amp;H71</f>
         <v/>
       </c>
@@ -3052,7 +3085,7 @@
       <c r="F72" s="10"/>
       <c r="G72" s="10"/>
       <c r="H72" s="10"/>
-      <c r="I72" s="13" t="str">
+      <c r="I72" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A72,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B72,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C72,Lists!$D:$E,2,0),""),D72,E72,F72,IF(G72="","",TEXT(G72,"00")))&amp;H72</f>
         <v/>
       </c>
@@ -3066,7 +3099,7 @@
       <c r="F73" s="10"/>
       <c r="G73" s="10"/>
       <c r="H73" s="10"/>
-      <c r="I73" s="13" t="str">
+      <c r="I73" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A73,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B73,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C73,Lists!$D:$E,2,0),""),D73,E73,F73,IF(G73="","",TEXT(G73,"00")))&amp;H73</f>
         <v/>
       </c>
@@ -3080,7 +3113,7 @@
       <c r="F74" s="10"/>
       <c r="G74" s="10"/>
       <c r="H74" s="10"/>
-      <c r="I74" s="13" t="str">
+      <c r="I74" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A74,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B74,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C74,Lists!$D:$E,2,0),""),D74,E74,F74,IF(G74="","",TEXT(G74,"00")))&amp;H74</f>
         <v/>
       </c>
@@ -3094,7 +3127,7 @@
       <c r="F75" s="10"/>
       <c r="G75" s="10"/>
       <c r="H75" s="10"/>
-      <c r="I75" s="13" t="str">
+      <c r="I75" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A75,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B75,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C75,Lists!$D:$E,2,0),""),D75,E75,F75,IF(G75="","",TEXT(G75,"00")))&amp;H75</f>
         <v/>
       </c>
@@ -3108,7 +3141,7 @@
       <c r="F76" s="10"/>
       <c r="G76" s="10"/>
       <c r="H76" s="10"/>
-      <c r="I76" s="13" t="str">
+      <c r="I76" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A76,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B76,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C76,Lists!$D:$E,2,0),""),D76,E76,F76,IF(G76="","",TEXT(G76,"00")))&amp;H76</f>
         <v/>
       </c>
@@ -3122,7 +3155,7 @@
       <c r="F77" s="10"/>
       <c r="G77" s="10"/>
       <c r="H77" s="10"/>
-      <c r="I77" s="13" t="str">
+      <c r="I77" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A77,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B77,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C77,Lists!$D:$E,2,0),""),D77,E77,F77,IF(G77="","",TEXT(G77,"00")))&amp;H77</f>
         <v/>
       </c>
@@ -3136,7 +3169,7 @@
       <c r="F78" s="10"/>
       <c r="G78" s="10"/>
       <c r="H78" s="10"/>
-      <c r="I78" s="13" t="str">
+      <c r="I78" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A78,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B78,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C78,Lists!$D:$E,2,0),""),D78,E78,F78,IF(G78="","",TEXT(G78,"00")))&amp;H78</f>
         <v/>
       </c>
@@ -3150,7 +3183,7 @@
       <c r="F79" s="10"/>
       <c r="G79" s="10"/>
       <c r="H79" s="10"/>
-      <c r="I79" s="13" t="str">
+      <c r="I79" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A79,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B79,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C79,Lists!$D:$E,2,0),""),D79,E79,F79,IF(G79="","",TEXT(G79,"00")))&amp;H79</f>
         <v/>
       </c>
@@ -3164,7 +3197,7 @@
       <c r="F80" s="10"/>
       <c r="G80" s="10"/>
       <c r="H80" s="10"/>
-      <c r="I80" s="13" t="str">
+      <c r="I80" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A80,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B80,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C80,Lists!$D:$E,2,0),""),D80,E80,F80,IF(G80="","",TEXT(G80,"00")))&amp;H80</f>
         <v/>
       </c>
@@ -3178,7 +3211,7 @@
       <c r="F81" s="10"/>
       <c r="G81" s="10"/>
       <c r="H81" s="10"/>
-      <c r="I81" s="13" t="str">
+      <c r="I81" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A81,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B81,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C81,Lists!$D:$E,2,0),""),D81,E81,F81,IF(G81="","",TEXT(G81,"00")))&amp;H81</f>
         <v/>
       </c>
@@ -3192,7 +3225,7 @@
       <c r="F82" s="10"/>
       <c r="G82" s="10"/>
       <c r="H82" s="10"/>
-      <c r="I82" s="13" t="str">
+      <c r="I82" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A82,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B82,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C82,Lists!$D:$E,2,0),""),D82,E82,F82,IF(G82="","",TEXT(G82,"00")))&amp;H82</f>
         <v/>
       </c>
@@ -3206,7 +3239,7 @@
       <c r="F83" s="10"/>
       <c r="G83" s="10"/>
       <c r="H83" s="10"/>
-      <c r="I83" s="13" t="str">
+      <c r="I83" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A83,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B83,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C83,Lists!$D:$E,2,0),""),D83,E83,F83,IF(G83="","",TEXT(G83,"00")))&amp;H83</f>
         <v/>
       </c>
@@ -3220,7 +3253,7 @@
       <c r="F84" s="10"/>
       <c r="G84" s="10"/>
       <c r="H84" s="10"/>
-      <c r="I84" s="13" t="str">
+      <c r="I84" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A84,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B84,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C84,Lists!$D:$E,2,0),""),D84,E84,F84,IF(G84="","",TEXT(G84,"00")))&amp;H84</f>
         <v/>
       </c>
@@ -3234,7 +3267,7 @@
       <c r="F85" s="10"/>
       <c r="G85" s="10"/>
       <c r="H85" s="10"/>
-      <c r="I85" s="13" t="str">
+      <c r="I85" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A85,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B85,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C85,Lists!$D:$E,2,0),""),D85,E85,F85,IF(G85="","",TEXT(G85,"00")))&amp;H85</f>
         <v/>
       </c>
@@ -3248,7 +3281,7 @@
       <c r="F86" s="10"/>
       <c r="G86" s="10"/>
       <c r="H86" s="10"/>
-      <c r="I86" s="13" t="str">
+      <c r="I86" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A86,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B86,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C86,Lists!$D:$E,2,0),""),D86,E86,F86,IF(G86="","",TEXT(G86,"00")))&amp;H86</f>
         <v/>
       </c>
@@ -3262,7 +3295,7 @@
       <c r="F87" s="10"/>
       <c r="G87" s="10"/>
       <c r="H87" s="10"/>
-      <c r="I87" s="13" t="str">
+      <c r="I87" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A87,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B87,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C87,Lists!$D:$E,2,0),""),D87,E87,F87,IF(G87="","",TEXT(G87,"00")))&amp;H87</f>
         <v/>
       </c>
@@ -3276,7 +3309,7 @@
       <c r="F88" s="10"/>
       <c r="G88" s="10"/>
       <c r="H88" s="10"/>
-      <c r="I88" s="13" t="str">
+      <c r="I88" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A88,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B88,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C88,Lists!$D:$E,2,0),""),D88,E88,F88,IF(G88="","",TEXT(G88,"00")))&amp;H88</f>
         <v/>
       </c>
@@ -3290,7 +3323,7 @@
       <c r="F89" s="10"/>
       <c r="G89" s="10"/>
       <c r="H89" s="10"/>
-      <c r="I89" s="13" t="str">
+      <c r="I89" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A89,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B89,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C89,Lists!$D:$E,2,0),""),D89,E89,F89,IF(G89="","",TEXT(G89,"00")))&amp;H89</f>
         <v/>
       </c>
@@ -3304,7 +3337,7 @@
       <c r="F90" s="10"/>
       <c r="G90" s="10"/>
       <c r="H90" s="10"/>
-      <c r="I90" s="13" t="str">
+      <c r="I90" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A90,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B90,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C90,Lists!$D:$E,2,0),""),D90,E90,F90,IF(G90="","",TEXT(G90,"00")))&amp;H90</f>
         <v/>
       </c>
@@ -3318,7 +3351,7 @@
       <c r="F91" s="10"/>
       <c r="G91" s="10"/>
       <c r="H91" s="10"/>
-      <c r="I91" s="13" t="str">
+      <c r="I91" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A91,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B91,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C91,Lists!$D:$E,2,0),""),D91,E91,F91,IF(G91="","",TEXT(G91,"00")))&amp;H91</f>
         <v/>
       </c>
@@ -3332,7 +3365,7 @@
       <c r="F92" s="10"/>
       <c r="G92" s="10"/>
       <c r="H92" s="10"/>
-      <c r="I92" s="13" t="str">
+      <c r="I92" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A92,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B92,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C92,Lists!$D:$E,2,0),""),D92,E92,F92,IF(G92="","",TEXT(G92,"00")))&amp;H92</f>
         <v/>
       </c>
@@ -3346,7 +3379,7 @@
       <c r="F93" s="10"/>
       <c r="G93" s="10"/>
       <c r="H93" s="10"/>
-      <c r="I93" s="13" t="str">
+      <c r="I93" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A93,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B93,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C93,Lists!$D:$E,2,0),""),D93,E93,F93,IF(G93="","",TEXT(G93,"00")))&amp;H93</f>
         <v/>
       </c>
@@ -3360,7 +3393,7 @@
       <c r="F94" s="10"/>
       <c r="G94" s="10"/>
       <c r="H94" s="10"/>
-      <c r="I94" s="13" t="str">
+      <c r="I94" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A94,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B94,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C94,Lists!$D:$E,2,0),""),D94,E94,F94,IF(G94="","",TEXT(G94,"00")))&amp;H94</f>
         <v/>
       </c>
@@ -3374,7 +3407,7 @@
       <c r="F95" s="10"/>
       <c r="G95" s="10"/>
       <c r="H95" s="10"/>
-      <c r="I95" s="13" t="str">
+      <c r="I95" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A95,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B95,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C95,Lists!$D:$E,2,0),""),D95,E95,F95,IF(G95="","",TEXT(G95,"00")))&amp;H95</f>
         <v/>
       </c>
@@ -3388,7 +3421,7 @@
       <c r="F96" s="10"/>
       <c r="G96" s="10"/>
       <c r="H96" s="10"/>
-      <c r="I96" s="13" t="str">
+      <c r="I96" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A96,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B96,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C96,Lists!$D:$E,2,0),""),D96,E96,F96,IF(G96="","",TEXT(G96,"00")))&amp;H96</f>
         <v/>
       </c>
@@ -3402,7 +3435,7 @@
       <c r="F97" s="10"/>
       <c r="G97" s="10"/>
       <c r="H97" s="10"/>
-      <c r="I97" s="13" t="str">
+      <c r="I97" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A97,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B97,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C97,Lists!$D:$E,2,0),""),D97,E97,F97,IF(G97="","",TEXT(G97,"00")))&amp;H97</f>
         <v/>
       </c>
@@ -3416,7 +3449,7 @@
       <c r="F98" s="10"/>
       <c r="G98" s="10"/>
       <c r="H98" s="10"/>
-      <c r="I98" s="13" t="str">
+      <c r="I98" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A98,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B98,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C98,Lists!$D:$E,2,0),""),D98,E98,F98,IF(G98="","",TEXT(G98,"00")))&amp;H98</f>
         <v/>
       </c>
@@ -3430,7 +3463,7 @@
       <c r="F99" s="10"/>
       <c r="G99" s="10"/>
       <c r="H99" s="10"/>
-      <c r="I99" s="13" t="str">
+      <c r="I99" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A99,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B99,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C99,Lists!$D:$E,2,0),""),D99,E99,F99,IF(G99="","",TEXT(G99,"00")))&amp;H99</f>
         <v/>
       </c>
@@ -3444,7 +3477,7 @@
       <c r="F100" s="10"/>
       <c r="G100" s="10"/>
       <c r="H100" s="10"/>
-      <c r="I100" s="13" t="str">
+      <c r="I100" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A100,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B100,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C100,Lists!$D:$E,2,0),""),D100,E100,F100,IF(G100="","",TEXT(G100,"00")))&amp;H100</f>
         <v/>
       </c>
@@ -3458,7 +3491,7 @@
       <c r="F101" s="10"/>
       <c r="G101" s="10"/>
       <c r="H101" s="10"/>
-      <c r="I101" s="13" t="str">
+      <c r="I101" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A101,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B101,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C101,Lists!$D:$E,2,0),""),D101,E101,F101,IF(G101="","",TEXT(G101,"00")))&amp;H101</f>
         <v/>
       </c>
@@ -3472,7 +3505,7 @@
       <c r="F102" s="10"/>
       <c r="G102" s="10"/>
       <c r="H102" s="10"/>
-      <c r="I102" s="13" t="str">
+      <c r="I102" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A102,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B102,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C102,Lists!$D:$E,2,0),""),D102,E102,F102,IF(G102="","",TEXT(G102,"00")))&amp;H102</f>
         <v/>
       </c>
@@ -3486,7 +3519,7 @@
       <c r="F103" s="10"/>
       <c r="G103" s="10"/>
       <c r="H103" s="10"/>
-      <c r="I103" s="13" t="str">
+      <c r="I103" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A103,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B103,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C103,Lists!$D:$E,2,0),""),D103,E103,F103,IF(G103="","",TEXT(G103,"00")))&amp;H103</f>
         <v/>
       </c>
@@ -3500,7 +3533,7 @@
       <c r="F104" s="10"/>
       <c r="G104" s="10"/>
       <c r="H104" s="10"/>
-      <c r="I104" s="13" t="str">
+      <c r="I104" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A104,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B104,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C104,Lists!$D:$E,2,0),""),D104,E104,F104,IF(G104="","",TEXT(G104,"00")))&amp;H104</f>
         <v/>
       </c>
@@ -3514,7 +3547,7 @@
       <c r="F105" s="10"/>
       <c r="G105" s="10"/>
       <c r="H105" s="10"/>
-      <c r="I105" s="13" t="str">
+      <c r="I105" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A105,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B105,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C105,Lists!$D:$E,2,0),""),D105,E105,F105,IF(G105="","",TEXT(G105,"00")))&amp;H105</f>
         <v/>
       </c>
@@ -3528,7 +3561,7 @@
       <c r="F106" s="10"/>
       <c r="G106" s="10"/>
       <c r="H106" s="10"/>
-      <c r="I106" s="13" t="str">
+      <c r="I106" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A106,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B106,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C106,Lists!$D:$E,2,0),""),D106,E106,F106,IF(G106="","",TEXT(G106,"00")))&amp;H106</f>
         <v/>
       </c>
@@ -3542,7 +3575,7 @@
       <c r="F107" s="10"/>
       <c r="G107" s="10"/>
       <c r="H107" s="10"/>
-      <c r="I107" s="13" t="str">
+      <c r="I107" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A107,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B107,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C107,Lists!$D:$E,2,0),""),D107,E107,F107,IF(G107="","",TEXT(G107,"00")))&amp;H107</f>
         <v/>
       </c>
@@ -3556,7 +3589,7 @@
       <c r="F108" s="10"/>
       <c r="G108" s="10"/>
       <c r="H108" s="10"/>
-      <c r="I108" s="13" t="str">
+      <c r="I108" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A108,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B108,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C108,Lists!$D:$E,2,0),""),D108,E108,F108,IF(G108="","",TEXT(G108,"00")))&amp;H108</f>
         <v/>
       </c>
@@ -3570,7 +3603,7 @@
       <c r="F109" s="10"/>
       <c r="G109" s="10"/>
       <c r="H109" s="10"/>
-      <c r="I109" s="13" t="str">
+      <c r="I109" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A109,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B109,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C109,Lists!$D:$E,2,0),""),D109,E109,F109,IF(G109="","",TEXT(G109,"00")))&amp;H109</f>
         <v/>
       </c>
@@ -3584,7 +3617,7 @@
       <c r="F110" s="10"/>
       <c r="G110" s="10"/>
       <c r="H110" s="10"/>
-      <c r="I110" s="13" t="str">
+      <c r="I110" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A110,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B110,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C110,Lists!$D:$E,2,0),""),D110,E110,F110,IF(G110="","",TEXT(G110,"00")))&amp;H110</f>
         <v/>
       </c>
@@ -3598,7 +3631,7 @@
       <c r="F111" s="10"/>
       <c r="G111" s="10"/>
       <c r="H111" s="10"/>
-      <c r="I111" s="13" t="str">
+      <c r="I111" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A111,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B111,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C111,Lists!$D:$E,2,0),""),D111,E111,F111,IF(G111="","",TEXT(G111,"00")))&amp;H111</f>
         <v/>
       </c>
@@ -3612,7 +3645,7 @@
       <c r="F112" s="10"/>
       <c r="G112" s="10"/>
       <c r="H112" s="10"/>
-      <c r="I112" s="13" t="str">
+      <c r="I112" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A112,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B112,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C112,Lists!$D:$E,2,0),""),D112,E112,F112,IF(G112="","",TEXT(G112,"00")))&amp;H112</f>
         <v/>
       </c>
@@ -3626,7 +3659,7 @@
       <c r="F113" s="10"/>
       <c r="G113" s="10"/>
       <c r="H113" s="10"/>
-      <c r="I113" s="13" t="str">
+      <c r="I113" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A113,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B113,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C113,Lists!$D:$E,2,0),""),D113,E113,F113,IF(G113="","",TEXT(G113,"00")))&amp;H113</f>
         <v/>
       </c>
@@ -3640,7 +3673,7 @@
       <c r="F114" s="10"/>
       <c r="G114" s="10"/>
       <c r="H114" s="10"/>
-      <c r="I114" s="13" t="str">
+      <c r="I114" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A114,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B114,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C114,Lists!$D:$E,2,0),""),D114,E114,F114,IF(G114="","",TEXT(G114,"00")))&amp;H114</f>
         <v/>
       </c>
@@ -3654,7 +3687,7 @@
       <c r="F115" s="10"/>
       <c r="G115" s="10"/>
       <c r="H115" s="10"/>
-      <c r="I115" s="13" t="str">
+      <c r="I115" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A115,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B115,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C115,Lists!$D:$E,2,0),""),D115,E115,F115,IF(G115="","",TEXT(G115,"00")))&amp;H115</f>
         <v/>
       </c>
@@ -3668,7 +3701,7 @@
       <c r="F116" s="10"/>
       <c r="G116" s="10"/>
       <c r="H116" s="10"/>
-      <c r="I116" s="13" t="str">
+      <c r="I116" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A116,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B116,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C116,Lists!$D:$E,2,0),""),D116,E116,F116,IF(G116="","",TEXT(G116,"00")))&amp;H116</f>
         <v/>
       </c>
@@ -3682,7 +3715,7 @@
       <c r="F117" s="10"/>
       <c r="G117" s="10"/>
       <c r="H117" s="10"/>
-      <c r="I117" s="13" t="str">
+      <c r="I117" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A117,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B117,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C117,Lists!$D:$E,2,0),""),D117,E117,F117,IF(G117="","",TEXT(G117,"00")))&amp;H117</f>
         <v/>
       </c>
@@ -3696,7 +3729,7 @@
       <c r="F118" s="10"/>
       <c r="G118" s="10"/>
       <c r="H118" s="10"/>
-      <c r="I118" s="13" t="str">
+      <c r="I118" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A118,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B118,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C118,Lists!$D:$E,2,0),""),D118,E118,F118,IF(G118="","",TEXT(G118,"00")))&amp;H118</f>
         <v/>
       </c>
@@ -3710,7 +3743,7 @@
       <c r="F119" s="10"/>
       <c r="G119" s="10"/>
       <c r="H119" s="10"/>
-      <c r="I119" s="13" t="str">
+      <c r="I119" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A119,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B119,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C119,Lists!$D:$E,2,0),""),D119,E119,F119,IF(G119="","",TEXT(G119,"00")))&amp;H119</f>
         <v/>
       </c>
@@ -3724,7 +3757,7 @@
       <c r="F120" s="10"/>
       <c r="G120" s="10"/>
       <c r="H120" s="10"/>
-      <c r="I120" s="13" t="str">
+      <c r="I120" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A120,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B120,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C120,Lists!$D:$E,2,0),""),D120,E120,F120,IF(G120="","",TEXT(G120,"00")))&amp;H120</f>
         <v/>
       </c>
@@ -3738,7 +3771,7 @@
       <c r="F121" s="10"/>
       <c r="G121" s="10"/>
       <c r="H121" s="10"/>
-      <c r="I121" s="13" t="str">
+      <c r="I121" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A121,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B121,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C121,Lists!$D:$E,2,0),""),D121,E121,F121,IF(G121="","",TEXT(G121,"00")))&amp;H121</f>
         <v/>
       </c>
@@ -3752,7 +3785,7 @@
       <c r="F122" s="10"/>
       <c r="G122" s="10"/>
       <c r="H122" s="10"/>
-      <c r="I122" s="13" t="str">
+      <c r="I122" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A122,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B122,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C122,Lists!$D:$E,2,0),""),D122,E122,F122,IF(G122="","",TEXT(G122,"00")))&amp;H122</f>
         <v/>
       </c>
@@ -3766,7 +3799,7 @@
       <c r="F123" s="10"/>
       <c r="G123" s="10"/>
       <c r="H123" s="10"/>
-      <c r="I123" s="13" t="str">
+      <c r="I123" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A123,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B123,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C123,Lists!$D:$E,2,0),""),D123,E123,F123,IF(G123="","",TEXT(G123,"00")))&amp;H123</f>
         <v/>
       </c>
@@ -3780,7 +3813,7 @@
       <c r="F124" s="10"/>
       <c r="G124" s="10"/>
       <c r="H124" s="10"/>
-      <c r="I124" s="13" t="str">
+      <c r="I124" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A124,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B124,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C124,Lists!$D:$E,2,0),""),D124,E124,F124,IF(G124="","",TEXT(G124,"00")))&amp;H124</f>
         <v/>
       </c>
@@ -3794,7 +3827,7 @@
       <c r="F125" s="10"/>
       <c r="G125" s="10"/>
       <c r="H125" s="10"/>
-      <c r="I125" s="13" t="str">
+      <c r="I125" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A125,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B125,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C125,Lists!$D:$E,2,0),""),D125,E125,F125,IF(G125="","",TEXT(G125,"00")))&amp;H125</f>
         <v/>
       </c>
@@ -3808,7 +3841,7 @@
       <c r="F126" s="10"/>
       <c r="G126" s="10"/>
       <c r="H126" s="10"/>
-      <c r="I126" s="13" t="str">
+      <c r="I126" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A126,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B126,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C126,Lists!$D:$E,2,0),""),D126,E126,F126,IF(G126="","",TEXT(G126,"00")))&amp;H126</f>
         <v/>
       </c>
@@ -3822,7 +3855,7 @@
       <c r="F127" s="10"/>
       <c r="G127" s="10"/>
       <c r="H127" s="10"/>
-      <c r="I127" s="13" t="str">
+      <c r="I127" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A127,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B127,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C127,Lists!$D:$E,2,0),""),D127,E127,F127,IF(G127="","",TEXT(G127,"00")))&amp;H127</f>
         <v/>
       </c>
@@ -3836,7 +3869,7 @@
       <c r="F128" s="10"/>
       <c r="G128" s="10"/>
       <c r="H128" s="10"/>
-      <c r="I128" s="13" t="str">
+      <c r="I128" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A128,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B128,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C128,Lists!$D:$E,2,0),""),D128,E128,F128,IF(G128="","",TEXT(G128,"00")))&amp;H128</f>
         <v/>
       </c>
@@ -3850,7 +3883,7 @@
       <c r="F129" s="10"/>
       <c r="G129" s="10"/>
       <c r="H129" s="10"/>
-      <c r="I129" s="13" t="str">
+      <c r="I129" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A129,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B129,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C129,Lists!$D:$E,2,0),""),D129,E129,F129,IF(G129="","",TEXT(G129,"00")))&amp;H129</f>
         <v/>
       </c>
@@ -3864,7 +3897,7 @@
       <c r="F130" s="10"/>
       <c r="G130" s="10"/>
       <c r="H130" s="10"/>
-      <c r="I130" s="13" t="str">
+      <c r="I130" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A130,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B130,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C130,Lists!$D:$E,2,0),""),D130,E130,F130,IF(G130="","",TEXT(G130,"00")))&amp;H130</f>
         <v/>
       </c>
@@ -3878,7 +3911,7 @@
       <c r="F131" s="10"/>
       <c r="G131" s="10"/>
       <c r="H131" s="10"/>
-      <c r="I131" s="13" t="str">
+      <c r="I131" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A131,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B131,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C131,Lists!$D:$E,2,0),""),D131,E131,F131,IF(G131="","",TEXT(G131,"00")))&amp;H131</f>
         <v/>
       </c>
@@ -3892,7 +3925,7 @@
       <c r="F132" s="10"/>
       <c r="G132" s="10"/>
       <c r="H132" s="10"/>
-      <c r="I132" s="13" t="str">
+      <c r="I132" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A132,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B132,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C132,Lists!$D:$E,2,0),""),D132,E132,F132,IF(G132="","",TEXT(G132,"00")))&amp;H132</f>
         <v/>
       </c>
@@ -3906,7 +3939,7 @@
       <c r="F133" s="10"/>
       <c r="G133" s="10"/>
       <c r="H133" s="10"/>
-      <c r="I133" s="13" t="str">
+      <c r="I133" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A133,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B133,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C133,Lists!$D:$E,2,0),""),D133,E133,F133,IF(G133="","",TEXT(G133,"00")))&amp;H133</f>
         <v/>
       </c>
@@ -3920,7 +3953,7 @@
       <c r="F134" s="10"/>
       <c r="G134" s="10"/>
       <c r="H134" s="10"/>
-      <c r="I134" s="13" t="str">
+      <c r="I134" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A134,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B134,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C134,Lists!$D:$E,2,0),""),D134,E134,F134,IF(G134="","",TEXT(G134,"00")))&amp;H134</f>
         <v/>
       </c>
@@ -3934,7 +3967,7 @@
       <c r="F135" s="10"/>
       <c r="G135" s="10"/>
       <c r="H135" s="10"/>
-      <c r="I135" s="13" t="str">
+      <c r="I135" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A135,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B135,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C135,Lists!$D:$E,2,0),""),D135,E135,F135,IF(G135="","",TEXT(G135,"00")))&amp;H135</f>
         <v/>
       </c>
@@ -3948,7 +3981,7 @@
       <c r="F136" s="10"/>
       <c r="G136" s="10"/>
       <c r="H136" s="10"/>
-      <c r="I136" s="13" t="str">
+      <c r="I136" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A136,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B136,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C136,Lists!$D:$E,2,0),""),D136,E136,F136,IF(G136="","",TEXT(G136,"00")))&amp;H136</f>
         <v/>
       </c>
@@ -3962,7 +3995,7 @@
       <c r="F137" s="10"/>
       <c r="G137" s="10"/>
       <c r="H137" s="10"/>
-      <c r="I137" s="13" t="str">
+      <c r="I137" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A137,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B137,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C137,Lists!$D:$E,2,0),""),D137,E137,F137,IF(G137="","",TEXT(G137,"00")))&amp;H137</f>
         <v/>
       </c>
@@ -3976,7 +4009,7 @@
       <c r="F138" s="10"/>
       <c r="G138" s="10"/>
       <c r="H138" s="10"/>
-      <c r="I138" s="13" t="str">
+      <c r="I138" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A138,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B138,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C138,Lists!$D:$E,2,0),""),D138,E138,F138,IF(G138="","",TEXT(G138,"00")))&amp;H138</f>
         <v/>
       </c>
@@ -3990,7 +4023,7 @@
       <c r="F139" s="10"/>
       <c r="G139" s="10"/>
       <c r="H139" s="10"/>
-      <c r="I139" s="13" t="str">
+      <c r="I139" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A139,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B139,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C139,Lists!$D:$E,2,0),""),D139,E139,F139,IF(G139="","",TEXT(G139,"00")))&amp;H139</f>
         <v/>
       </c>
@@ -4004,7 +4037,7 @@
       <c r="F140" s="10"/>
       <c r="G140" s="10"/>
       <c r="H140" s="10"/>
-      <c r="I140" s="13" t="str">
+      <c r="I140" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A140,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B140,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C140,Lists!$D:$E,2,0),""),D140,E140,F140,IF(G140="","",TEXT(G140,"00")))&amp;H140</f>
         <v/>
       </c>
@@ -4018,7 +4051,7 @@
       <c r="F141" s="10"/>
       <c r="G141" s="10"/>
       <c r="H141" s="10"/>
-      <c r="I141" s="13" t="str">
+      <c r="I141" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A141,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B141,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C141,Lists!$D:$E,2,0),""),D141,E141,F141,IF(G141="","",TEXT(G141,"00")))&amp;H141</f>
         <v/>
       </c>
@@ -4032,7 +4065,7 @@
       <c r="F142" s="10"/>
       <c r="G142" s="10"/>
       <c r="H142" s="10"/>
-      <c r="I142" s="13" t="str">
+      <c r="I142" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A142,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B142,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C142,Lists!$D:$E,2,0),""),D142,E142,F142,IF(G142="","",TEXT(G142,"00")))&amp;H142</f>
         <v/>
       </c>
@@ -4046,7 +4079,7 @@
       <c r="F143" s="10"/>
       <c r="G143" s="10"/>
       <c r="H143" s="10"/>
-      <c r="I143" s="13" t="str">
+      <c r="I143" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A143,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B143,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C143,Lists!$D:$E,2,0),""),D143,E143,F143,IF(G143="","",TEXT(G143,"00")))&amp;H143</f>
         <v/>
       </c>
@@ -4060,7 +4093,7 @@
       <c r="F144" s="10"/>
       <c r="G144" s="10"/>
       <c r="H144" s="10"/>
-      <c r="I144" s="13" t="str">
+      <c r="I144" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A144,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B144,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C144,Lists!$D:$E,2,0),""),D144,E144,F144,IF(G144="","",TEXT(G144,"00")))&amp;H144</f>
         <v/>
       </c>
@@ -4074,7 +4107,7 @@
       <c r="F145" s="10"/>
       <c r="G145" s="10"/>
       <c r="H145" s="10"/>
-      <c r="I145" s="13" t="str">
+      <c r="I145" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A145,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B145,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C145,Lists!$D:$E,2,0),""),D145,E145,F145,IF(G145="","",TEXT(G145,"00")))&amp;H145</f>
         <v/>
       </c>
@@ -4088,7 +4121,7 @@
       <c r="F146" s="10"/>
       <c r="G146" s="10"/>
       <c r="H146" s="10"/>
-      <c r="I146" s="13" t="str">
+      <c r="I146" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A146,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B146,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C146,Lists!$D:$E,2,0),""),D146,E146,F146,IF(G146="","",TEXT(G146,"00")))&amp;H146</f>
         <v/>
       </c>
@@ -4102,7 +4135,7 @@
       <c r="F147" s="10"/>
       <c r="G147" s="10"/>
       <c r="H147" s="10"/>
-      <c r="I147" s="13" t="str">
+      <c r="I147" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A147,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B147,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C147,Lists!$D:$E,2,0),""),D147,E147,F147,IF(G147="","",TEXT(G147,"00")))&amp;H147</f>
         <v/>
       </c>
@@ -4116,7 +4149,7 @@
       <c r="F148" s="10"/>
       <c r="G148" s="10"/>
       <c r="H148" s="10"/>
-      <c r="I148" s="13" t="str">
+      <c r="I148" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A148,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B148,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C148,Lists!$D:$E,2,0),""),D148,E148,F148,IF(G148="","",TEXT(G148,"00")))&amp;H148</f>
         <v/>
       </c>
@@ -4130,7 +4163,7 @@
       <c r="F149" s="10"/>
       <c r="G149" s="10"/>
       <c r="H149" s="10"/>
-      <c r="I149" s="13" t="str">
+      <c r="I149" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A149,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B149,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C149,Lists!$D:$E,2,0),""),D149,E149,F149,IF(G149="","",TEXT(G149,"00")))&amp;H149</f>
         <v/>
       </c>
@@ -4144,7 +4177,7 @@
       <c r="F150" s="10"/>
       <c r="G150" s="10"/>
       <c r="H150" s="10"/>
-      <c r="I150" s="13" t="str">
+      <c r="I150" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A150,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B150,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C150,Lists!$D:$E,2,0),""),D150,E150,F150,IF(G150="","",TEXT(G150,"00")))&amp;H150</f>
         <v/>
       </c>
@@ -4158,7 +4191,7 @@
       <c r="F151" s="10"/>
       <c r="G151" s="10"/>
       <c r="H151" s="10"/>
-      <c r="I151" s="13" t="str">
+      <c r="I151" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A151,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B151,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C151,Lists!$D:$E,2,0),""),D151,E151,F151,IF(G151="","",TEXT(G151,"00")))&amp;H151</f>
         <v/>
       </c>
@@ -4172,7 +4205,7 @@
       <c r="F152" s="10"/>
       <c r="G152" s="10"/>
       <c r="H152" s="10"/>
-      <c r="I152" s="13" t="str">
+      <c r="I152" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A152,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B152,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C152,Lists!$D:$E,2,0),""),D152,E152,F152,IF(G152="","",TEXT(G152,"00")))&amp;H152</f>
         <v/>
       </c>
@@ -4186,7 +4219,7 @@
       <c r="F153" s="10"/>
       <c r="G153" s="10"/>
       <c r="H153" s="10"/>
-      <c r="I153" s="13" t="str">
+      <c r="I153" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A153,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B153,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C153,Lists!$D:$E,2,0),""),D153,E153,F153,IF(G153="","",TEXT(G153,"00")))&amp;H153</f>
         <v/>
       </c>
@@ -4200,7 +4233,7 @@
       <c r="F154" s="10"/>
       <c r="G154" s="10"/>
       <c r="H154" s="10"/>
-      <c r="I154" s="13" t="str">
+      <c r="I154" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A154,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B154,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C154,Lists!$D:$E,2,0),""),D154,E154,F154,IF(G154="","",TEXT(G154,"00")))&amp;H154</f>
         <v/>
       </c>
@@ -4214,7 +4247,7 @@
       <c r="F155" s="10"/>
       <c r="G155" s="10"/>
       <c r="H155" s="10"/>
-      <c r="I155" s="13" t="str">
+      <c r="I155" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A155,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B155,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C155,Lists!$D:$E,2,0),""),D155,E155,F155,IF(G155="","",TEXT(G155,"00")))&amp;H155</f>
         <v/>
       </c>
@@ -4228,7 +4261,7 @@
       <c r="F156" s="10"/>
       <c r="G156" s="10"/>
       <c r="H156" s="10"/>
-      <c r="I156" s="13" t="str">
+      <c r="I156" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A156,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B156,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C156,Lists!$D:$E,2,0),""),D156,E156,F156,IF(G156="","",TEXT(G156,"00")))&amp;H156</f>
         <v/>
       </c>
@@ -4242,7 +4275,7 @@
       <c r="F157" s="10"/>
       <c r="G157" s="10"/>
       <c r="H157" s="10"/>
-      <c r="I157" s="13" t="str">
+      <c r="I157" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A157,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B157,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C157,Lists!$D:$E,2,0),""),D157,E157,F157,IF(G157="","",TEXT(G157,"00")))&amp;H157</f>
         <v/>
       </c>
@@ -4256,7 +4289,7 @@
       <c r="F158" s="10"/>
       <c r="G158" s="10"/>
       <c r="H158" s="10"/>
-      <c r="I158" s="13" t="str">
+      <c r="I158" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A158,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B158,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C158,Lists!$D:$E,2,0),""),D158,E158,F158,IF(G158="","",TEXT(G158,"00")))&amp;H158</f>
         <v/>
       </c>
@@ -4270,7 +4303,7 @@
       <c r="F159" s="10"/>
       <c r="G159" s="10"/>
       <c r="H159" s="10"/>
-      <c r="I159" s="13" t="str">
+      <c r="I159" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A159,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B159,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C159,Lists!$D:$E,2,0),""),D159,E159,F159,IF(G159="","",TEXT(G159,"00")))&amp;H159</f>
         <v/>
       </c>
@@ -4284,7 +4317,7 @@
       <c r="F160" s="10"/>
       <c r="G160" s="10"/>
       <c r="H160" s="10"/>
-      <c r="I160" s="13" t="str">
+      <c r="I160" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A160,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B160,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C160,Lists!$D:$E,2,0),""),D160,E160,F160,IF(G160="","",TEXT(G160,"00")))&amp;H160</f>
         <v/>
       </c>
@@ -4298,7 +4331,7 @@
       <c r="F161" s="10"/>
       <c r="G161" s="10"/>
       <c r="H161" s="10"/>
-      <c r="I161" s="13" t="str">
+      <c r="I161" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A161,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B161,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C161,Lists!$D:$E,2,0),""),D161,E161,F161,IF(G161="","",TEXT(G161,"00")))&amp;H161</f>
         <v/>
       </c>
@@ -4312,7 +4345,7 @@
       <c r="F162" s="10"/>
       <c r="G162" s="10"/>
       <c r="H162" s="10"/>
-      <c r="I162" s="13" t="str">
+      <c r="I162" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A162,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B162,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C162,Lists!$D:$E,2,0),""),D162,E162,F162,IF(G162="","",TEXT(G162,"00")))&amp;H162</f>
         <v/>
       </c>
@@ -4326,7 +4359,7 @@
       <c r="F163" s="10"/>
       <c r="G163" s="10"/>
       <c r="H163" s="10"/>
-      <c r="I163" s="13" t="str">
+      <c r="I163" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A163,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B163,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C163,Lists!$D:$E,2,0),""),D163,E163,F163,IF(G163="","",TEXT(G163,"00")))&amp;H163</f>
         <v/>
       </c>
@@ -4340,7 +4373,7 @@
       <c r="F164" s="10"/>
       <c r="G164" s="10"/>
       <c r="H164" s="10"/>
-      <c r="I164" s="13" t="str">
+      <c r="I164" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A164,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B164,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C164,Lists!$D:$E,2,0),""),D164,E164,F164,IF(G164="","",TEXT(G164,"00")))&amp;H164</f>
         <v/>
       </c>
@@ -4354,7 +4387,7 @@
       <c r="F165" s="10"/>
       <c r="G165" s="10"/>
       <c r="H165" s="10"/>
-      <c r="I165" s="13" t="str">
+      <c r="I165" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A165,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B165,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C165,Lists!$D:$E,2,0),""),D165,E165,F165,IF(G165="","",TEXT(G165,"00")))&amp;H165</f>
         <v/>
       </c>
@@ -4368,7 +4401,7 @@
       <c r="F166" s="10"/>
       <c r="G166" s="10"/>
       <c r="H166" s="10"/>
-      <c r="I166" s="13" t="str">
+      <c r="I166" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A166,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B166,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C166,Lists!$D:$E,2,0),""),D166,E166,F166,IF(G166="","",TEXT(G166,"00")))&amp;H166</f>
         <v/>
       </c>
@@ -4382,7 +4415,7 @@
       <c r="F167" s="10"/>
       <c r="G167" s="10"/>
       <c r="H167" s="10"/>
-      <c r="I167" s="13" t="str">
+      <c r="I167" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A167,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B167,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C167,Lists!$D:$E,2,0),""),D167,E167,F167,IF(G167="","",TEXT(G167,"00")))&amp;H167</f>
         <v/>
       </c>
@@ -4396,7 +4429,7 @@
       <c r="F168" s="10"/>
       <c r="G168" s="10"/>
       <c r="H168" s="10"/>
-      <c r="I168" s="13" t="str">
+      <c r="I168" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A168,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B168,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C168,Lists!$D:$E,2,0),""),D168,E168,F168,IF(G168="","",TEXT(G168,"00")))&amp;H168</f>
         <v/>
       </c>
@@ -4410,7 +4443,7 @@
       <c r="F169" s="10"/>
       <c r="G169" s="10"/>
       <c r="H169" s="10"/>
-      <c r="I169" s="13" t="str">
+      <c r="I169" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A169,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B169,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C169,Lists!$D:$E,2,0),""),D169,E169,F169,IF(G169="","",TEXT(G169,"00")))&amp;H169</f>
         <v/>
       </c>
@@ -4424,7 +4457,7 @@
       <c r="F170" s="10"/>
       <c r="G170" s="10"/>
       <c r="H170" s="10"/>
-      <c r="I170" s="13" t="str">
+      <c r="I170" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A170,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B170,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C170,Lists!$D:$E,2,0),""),D170,E170,F170,IF(G170="","",TEXT(G170,"00")))&amp;H170</f>
         <v/>
       </c>
@@ -4438,7 +4471,7 @@
       <c r="F171" s="10"/>
       <c r="G171" s="10"/>
       <c r="H171" s="10"/>
-      <c r="I171" s="13" t="str">
+      <c r="I171" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A171,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B171,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C171,Lists!$D:$E,2,0),""),D171,E171,F171,IF(G171="","",TEXT(G171,"00")))&amp;H171</f>
         <v/>
       </c>
@@ -4452,7 +4485,7 @@
       <c r="F172" s="10"/>
       <c r="G172" s="10"/>
       <c r="H172" s="10"/>
-      <c r="I172" s="13" t="str">
+      <c r="I172" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A172,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B172,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C172,Lists!$D:$E,2,0),""),D172,E172,F172,IF(G172="","",TEXT(G172,"00")))&amp;H172</f>
         <v/>
       </c>
@@ -4466,7 +4499,7 @@
       <c r="F173" s="10"/>
       <c r="G173" s="10"/>
       <c r="H173" s="10"/>
-      <c r="I173" s="13" t="str">
+      <c r="I173" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A173,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B173,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C173,Lists!$D:$E,2,0),""),D173,E173,F173,IF(G173="","",TEXT(G173,"00")))&amp;H173</f>
         <v/>
       </c>
@@ -4480,7 +4513,7 @@
       <c r="F174" s="10"/>
       <c r="G174" s="10"/>
       <c r="H174" s="10"/>
-      <c r="I174" s="13" t="str">
+      <c r="I174" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A174,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B174,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C174,Lists!$D:$E,2,0),""),D174,E174,F174,IF(G174="","",TEXT(G174,"00")))&amp;H174</f>
         <v/>
       </c>
@@ -4494,7 +4527,7 @@
       <c r="F175" s="10"/>
       <c r="G175" s="10"/>
       <c r="H175" s="10"/>
-      <c r="I175" s="13" t="str">
+      <c r="I175" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A175,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B175,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C175,Lists!$D:$E,2,0),""),D175,E175,F175,IF(G175="","",TEXT(G175,"00")))&amp;H175</f>
         <v/>
       </c>
@@ -4508,7 +4541,7 @@
       <c r="F176" s="10"/>
       <c r="G176" s="10"/>
       <c r="H176" s="10"/>
-      <c r="I176" s="13" t="str">
+      <c r="I176" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A176,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B176,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C176,Lists!$D:$E,2,0),""),D176,E176,F176,IF(G176="","",TEXT(G176,"00")))&amp;H176</f>
         <v/>
       </c>
@@ -4522,7 +4555,7 @@
       <c r="F177" s="10"/>
       <c r="G177" s="10"/>
       <c r="H177" s="10"/>
-      <c r="I177" s="13" t="str">
+      <c r="I177" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A177,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B177,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C177,Lists!$D:$E,2,0),""),D177,E177,F177,IF(G177="","",TEXT(G177,"00")))&amp;H177</f>
         <v/>
       </c>
@@ -4536,7 +4569,7 @@
       <c r="F178" s="10"/>
       <c r="G178" s="10"/>
       <c r="H178" s="10"/>
-      <c r="I178" s="13" t="str">
+      <c r="I178" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A178,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B178,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C178,Lists!$D:$E,2,0),""),D178,E178,F178,IF(G178="","",TEXT(G178,"00")))&amp;H178</f>
         <v/>
       </c>
@@ -4550,7 +4583,7 @@
       <c r="F179" s="10"/>
       <c r="G179" s="10"/>
       <c r="H179" s="10"/>
-      <c r="I179" s="13" t="str">
+      <c r="I179" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A179,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B179,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C179,Lists!$D:$E,2,0),""),D179,E179,F179,IF(G179="","",TEXT(G179,"00")))&amp;H179</f>
         <v/>
       </c>
@@ -4564,7 +4597,7 @@
       <c r="F180" s="10"/>
       <c r="G180" s="10"/>
       <c r="H180" s="10"/>
-      <c r="I180" s="13" t="str">
+      <c r="I180" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A180,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B180,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C180,Lists!$D:$E,2,0),""),D180,E180,F180,IF(G180="","",TEXT(G180,"00")))&amp;H180</f>
         <v/>
       </c>
@@ -4578,7 +4611,7 @@
       <c r="F181" s="10"/>
       <c r="G181" s="10"/>
       <c r="H181" s="10"/>
-      <c r="I181" s="13" t="str">
+      <c r="I181" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A181,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B181,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C181,Lists!$D:$E,2,0),""),D181,E181,F181,IF(G181="","",TEXT(G181,"00")))&amp;H181</f>
         <v/>
       </c>
@@ -4592,7 +4625,7 @@
       <c r="F182" s="10"/>
       <c r="G182" s="10"/>
       <c r="H182" s="10"/>
-      <c r="I182" s="13" t="str">
+      <c r="I182" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A182,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B182,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C182,Lists!$D:$E,2,0),""),D182,E182,F182,IF(G182="","",TEXT(G182,"00")))&amp;H182</f>
         <v/>
       </c>
@@ -4606,7 +4639,7 @@
       <c r="F183" s="10"/>
       <c r="G183" s="10"/>
       <c r="H183" s="10"/>
-      <c r="I183" s="13" t="str">
+      <c r="I183" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A183,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B183,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C183,Lists!$D:$E,2,0),""),D183,E183,F183,IF(G183="","",TEXT(G183,"00")))&amp;H183</f>
         <v/>
       </c>
@@ -4620,7 +4653,7 @@
       <c r="F184" s="10"/>
       <c r="G184" s="10"/>
       <c r="H184" s="10"/>
-      <c r="I184" s="13" t="str">
+      <c r="I184" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A184,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B184,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C184,Lists!$D:$E,2,0),""),D184,E184,F184,IF(G184="","",TEXT(G184,"00")))&amp;H184</f>
         <v/>
       </c>
@@ -4634,7 +4667,7 @@
       <c r="F185" s="10"/>
       <c r="G185" s="10"/>
       <c r="H185" s="10"/>
-      <c r="I185" s="13" t="str">
+      <c r="I185" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A185,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B185,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C185,Lists!$D:$E,2,0),""),D185,E185,F185,IF(G185="","",TEXT(G185,"00")))&amp;H185</f>
         <v/>
       </c>
@@ -4648,7 +4681,7 @@
       <c r="F186" s="10"/>
       <c r="G186" s="10"/>
       <c r="H186" s="10"/>
-      <c r="I186" s="13" t="str">
+      <c r="I186" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A186,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B186,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C186,Lists!$D:$E,2,0),""),D186,E186,F186,IF(G186="","",TEXT(G186,"00")))&amp;H186</f>
         <v/>
       </c>
@@ -4662,7 +4695,7 @@
       <c r="F187" s="10"/>
       <c r="G187" s="10"/>
       <c r="H187" s="10"/>
-      <c r="I187" s="13" t="str">
+      <c r="I187" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A187,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B187,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C187,Lists!$D:$E,2,0),""),D187,E187,F187,IF(G187="","",TEXT(G187,"00")))&amp;H187</f>
         <v/>
       </c>
@@ -4676,7 +4709,7 @@
       <c r="F188" s="10"/>
       <c r="G188" s="10"/>
       <c r="H188" s="10"/>
-      <c r="I188" s="13" t="str">
+      <c r="I188" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A188,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B188,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C188,Lists!$D:$E,2,0),""),D188,E188,F188,IF(G188="","",TEXT(G188,"00")))&amp;H188</f>
         <v/>
       </c>
@@ -4690,7 +4723,7 @@
       <c r="F189" s="10"/>
       <c r="G189" s="10"/>
       <c r="H189" s="10"/>
-      <c r="I189" s="13" t="str">
+      <c r="I189" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A189,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B189,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C189,Lists!$D:$E,2,0),""),D189,E189,F189,IF(G189="","",TEXT(G189,"00")))&amp;H189</f>
         <v/>
       </c>
@@ -4704,7 +4737,7 @@
       <c r="F190" s="10"/>
       <c r="G190" s="10"/>
       <c r="H190" s="10"/>
-      <c r="I190" s="13" t="str">
+      <c r="I190" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A190,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B190,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C190,Lists!$D:$E,2,0),""),D190,E190,F190,IF(G190="","",TEXT(G190,"00")))&amp;H190</f>
         <v/>
       </c>
@@ -4718,7 +4751,7 @@
       <c r="F191" s="10"/>
       <c r="G191" s="10"/>
       <c r="H191" s="10"/>
-      <c r="I191" s="13" t="str">
+      <c r="I191" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A191,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B191,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C191,Lists!$D:$E,2,0),""),D191,E191,F191,IF(G191="","",TEXT(G191,"00")))&amp;H191</f>
         <v/>
       </c>
@@ -4732,7 +4765,7 @@
       <c r="F192" s="10"/>
       <c r="G192" s="10"/>
       <c r="H192" s="10"/>
-      <c r="I192" s="13" t="str">
+      <c r="I192" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A192,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B192,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C192,Lists!$D:$E,2,0),""),D192,E192,F192,IF(G192="","",TEXT(G192,"00")))&amp;H192</f>
         <v/>
       </c>
@@ -4746,7 +4779,7 @@
       <c r="F193" s="10"/>
       <c r="G193" s="10"/>
       <c r="H193" s="10"/>
-      <c r="I193" s="13" t="str">
+      <c r="I193" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A193,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B193,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C193,Lists!$D:$E,2,0),""),D193,E193,F193,IF(G193="","",TEXT(G193,"00")))&amp;H193</f>
         <v/>
       </c>
@@ -4760,7 +4793,7 @@
       <c r="F194" s="10"/>
       <c r="G194" s="10"/>
       <c r="H194" s="10"/>
-      <c r="I194" s="13" t="str">
+      <c r="I194" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A194,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B194,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C194,Lists!$D:$E,2,0),""),D194,E194,F194,IF(G194="","",TEXT(G194,"00")))&amp;H194</f>
         <v/>
       </c>
@@ -4774,7 +4807,7 @@
       <c r="F195" s="10"/>
       <c r="G195" s="10"/>
       <c r="H195" s="10"/>
-      <c r="I195" s="13" t="str">
+      <c r="I195" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A195,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B195,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C195,Lists!$D:$E,2,0),""),D195,E195,F195,IF(G195="","",TEXT(G195,"00")))&amp;H195</f>
         <v/>
       </c>
@@ -4788,7 +4821,7 @@
       <c r="F196" s="10"/>
       <c r="G196" s="10"/>
       <c r="H196" s="10"/>
-      <c r="I196" s="13" t="str">
+      <c r="I196" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A196,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B196,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C196,Lists!$D:$E,2,0),""),D196,E196,F196,IF(G196="","",TEXT(G196,"00")))&amp;H196</f>
         <v/>
       </c>
@@ -4802,7 +4835,7 @@
       <c r="F197" s="10"/>
       <c r="G197" s="10"/>
       <c r="H197" s="10"/>
-      <c r="I197" s="13" t="str">
+      <c r="I197" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A197,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B197,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C197,Lists!$D:$E,2,0),""),D197,E197,F197,IF(G197="","",TEXT(G197,"00")))&amp;H197</f>
         <v/>
       </c>
@@ -4816,7 +4849,7 @@
       <c r="F198" s="10"/>
       <c r="G198" s="10"/>
       <c r="H198" s="10"/>
-      <c r="I198" s="13" t="str">
+      <c r="I198" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A198,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B198,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C198,Lists!$D:$E,2,0),""),D198,E198,F198,IF(G198="","",TEXT(G198,"00")))&amp;H198</f>
         <v/>
       </c>
@@ -4830,7 +4863,7 @@
       <c r="F199" s="10"/>
       <c r="G199" s="10"/>
       <c r="H199" s="10"/>
-      <c r="I199" s="13" t="str">
+      <c r="I199" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A199,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B199,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C199,Lists!$D:$E,2,0),""),D199,E199,F199,IF(G199="","",TEXT(G199,"00")))&amp;H199</f>
         <v/>
       </c>
@@ -4844,7 +4877,7 @@
       <c r="F200" s="10"/>
       <c r="G200" s="10"/>
       <c r="H200" s="10"/>
-      <c r="I200" s="13" t="str">
+      <c r="I200" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A200,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B200,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C200,Lists!$D:$E,2,0),""),D200,E200,F200,IF(G200="","",TEXT(G200,"00")))&amp;H200</f>
         <v/>
       </c>
@@ -4858,7 +4891,7 @@
       <c r="F201" s="10"/>
       <c r="G201" s="10"/>
       <c r="H201" s="10"/>
-      <c r="I201" s="13" t="str">
+      <c r="I201" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A201,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B201,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C201,Lists!$D:$E,2,0),""),D201,E201,F201,IF(G201="","",TEXT(G201,"00")))&amp;H201</f>
         <v/>
       </c>
@@ -4872,7 +4905,7 @@
       <c r="F202" s="10"/>
       <c r="G202" s="10"/>
       <c r="H202" s="10"/>
-      <c r="I202" s="13" t="str">
+      <c r="I202" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A202,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B202,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C202,Lists!$D:$E,2,0),""),D202,E202,F202,IF(G202="","",TEXT(G202,"00")))&amp;H202</f>
         <v/>
       </c>
@@ -4886,7 +4919,7 @@
       <c r="F203" s="10"/>
       <c r="G203" s="10"/>
       <c r="H203" s="10"/>
-      <c r="I203" s="13" t="str">
+      <c r="I203" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A203,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B203,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C203,Lists!$D:$E,2,0),""),D203,E203,F203,IF(G203="","",TEXT(G203,"00")))&amp;H203</f>
         <v/>
       </c>
@@ -4900,7 +4933,7 @@
       <c r="F204" s="10"/>
       <c r="G204" s="10"/>
       <c r="H204" s="10"/>
-      <c r="I204" s="13" t="str">
+      <c r="I204" s="15" t="str">
         <f>TEXTJOIN("-",TRUE(),IFERROR(VLOOKUP(A204,Lists!$A:$B,2,0),""),IFERROR(VLOOKUP(B204,Lists!$O:$P,2,0),""),IFERROR(VLOOKUP(C204,Lists!$D:$E,2,0),""),D204,E204,F204,IF(G204="","",TEXT(G204,"00")))&amp;H204</f>
         <v/>
       </c>
@@ -5758,554 +5791,601 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="D1" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1" s="3" t="s">
+      <c r="A1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="I1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K1" s="3" t="s">
+      <c r="D1" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E1" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="3" t="s">
+      <c r="G1" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="I1" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="K1" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="M1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="O1" s="5" t="s">
         <v>17</v>
       </c>
+      <c r="P1" s="5" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="E2" s="6"/>
-      <c r="G2" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="K2" s="6" t="s">
+      <c r="A2" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="4"/>
+      <c r="G2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I2" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="M2" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="O2" s="6" t="s">
+      <c r="K2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="P2" s="6"/>
+      <c r="O2" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="P2" s="4"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="G3" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="E3" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" s="6" t="s">
+      <c r="I3" s="4" t="s">
         <v>48</v>
       </c>
-      <c r="I3" s="6" t="s">
+      <c r="K3" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="M3" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="O3" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="P3" s="4" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="O4" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="P4" s="4" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="K3" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="M3" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="O3" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="P3" s="6" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="O4" s="6" t="s">
+      <c r="B5" s="4" t="s">
         <v>59</v>
       </c>
-      <c r="P4" s="6" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="s">
-        <v>38</v>
-      </c>
-      <c r="B5" s="6" t="s">
+      <c r="D5" s="4" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="G5" s="6" t="s">
+      <c r="E5" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="G5" s="4" t="s">
         <v>62</v>
       </c>
       <c r="O5" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="P5" s="11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D6" s="6" t="s">
+      <c r="E6" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="E6" s="6" t="s">
-        <v>71</v>
-      </c>
-      <c r="G6" s="6" t="s">
+      <c r="B7" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="G9" s="4"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="G10" s="4"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="G11" s="4"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="G12" s="4"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>98</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="G13" s="4"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="B17" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="E17" s="4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>116</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="E18" s="4" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="s">
+        <v>118</v>
+      </c>
+      <c r="B19" s="4" t="s">
+        <v>119</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>120</v>
+      </c>
+      <c r="E19" s="4" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>122</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="E20" s="4" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>125</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E21" s="4" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B22" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="E22" s="4" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>132</v>
+      </c>
+      <c r="E23" s="4" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="D24" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="E24" s="4" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="D25" s="4" t="s">
+        <v>135</v>
+      </c>
+      <c r="E25" s="4" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="D26" s="4" t="s">
+        <v>136</v>
+      </c>
+      <c r="E26" s="4" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="D27" s="4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E27" s="4" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="D28" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="E28" s="4" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="29" ht="15.75" customHeight="1">
+      <c r="D29" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="E29" s="4" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="30" ht="15.75" customHeight="1">
+      <c r="D30" s="4" t="s">
+        <v>141</v>
+      </c>
+      <c r="E30" s="4" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="31" ht="15.75" customHeight="1">
+      <c r="D31" s="4" t="s">
+        <v>142</v>
+      </c>
+      <c r="E31" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="32" ht="15.75" customHeight="1">
+      <c r="D32" s="4" t="s">
+        <v>143</v>
+      </c>
+      <c r="E32" s="4" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="33" ht="15.75" customHeight="1">
+      <c r="D33" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="E33" s="4" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="34" ht="15.75" customHeight="1">
+      <c r="D34" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E34" s="4" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="35" ht="15.75" customHeight="1">
+      <c r="D35" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="E35" s="4" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="36" ht="15.75" customHeight="1">
+      <c r="D36" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="E36" s="4" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="37" ht="15.75" customHeight="1">
+      <c r="D37" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="E37" s="4" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="38" ht="15.75" customHeight="1">
+      <c r="D38" s="4" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>74</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>75</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>78</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>80</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>81</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>84</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>85</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>86</v>
-      </c>
-      <c r="G9" s="6"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="s">
-        <v>87</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>88</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="G10" s="6"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="s">
-        <v>91</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>92</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>93</v>
-      </c>
-      <c r="G11" s="6"/>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="E12" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="G12" s="6"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="E13" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="G13" s="6"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>102</v>
-      </c>
-      <c r="E14" s="6" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="6" t="s">
-        <v>104</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>105</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>106</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="s">
-        <v>108</v>
-      </c>
-      <c r="B16" s="6" t="s">
-        <v>109</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>110</v>
-      </c>
-      <c r="E16" s="6" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="s">
-        <v>112</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>113</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="E17" s="6" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="s">
-        <v>115</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>116</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="E18" s="6" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>118</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>119</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>120</v>
-      </c>
-      <c r="E19" s="6" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="s">
-        <v>121</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>122</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>123</v>
-      </c>
-      <c r="E20" s="6" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="21" ht="15.75" customHeight="1">
-      <c r="A21" s="6" t="s">
-        <v>124</v>
-      </c>
-      <c r="B21" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="22" ht="15.75" customHeight="1">
-      <c r="A22" s="6" t="s">
-        <v>127</v>
-      </c>
-      <c r="B22" s="6" t="s">
-        <v>128</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="23" ht="15.75" customHeight="1">
-      <c r="A23" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="B23" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="E23" s="6" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="24" ht="15.75" customHeight="1">
-      <c r="D24" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="E24" s="6" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="25" ht="15.75" customHeight="1">
-      <c r="D25" s="6" t="s">
-        <v>135</v>
-      </c>
-      <c r="E25" s="6" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="26" ht="15.75" customHeight="1">
-      <c r="D26" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="E26" s="6" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="27" ht="15.75" customHeight="1">
-      <c r="D27" s="6" t="s">
-        <v>137</v>
-      </c>
-      <c r="E27" s="6" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="28" ht="15.75" customHeight="1">
-      <c r="D28" s="6" t="s">
-        <v>138</v>
-      </c>
-      <c r="E28" s="6" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="29" ht="15.75" customHeight="1">
-      <c r="D29" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="E29" s="6" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="30" ht="15.75" customHeight="1">
-      <c r="D30" s="6" t="s">
-        <v>141</v>
-      </c>
-      <c r="E30" s="6" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="31" ht="15.75" customHeight="1">
-      <c r="D31" s="6" t="s">
-        <v>142</v>
-      </c>
-      <c r="E31" s="6" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="32" ht="15.75" customHeight="1">
-      <c r="D32" s="6" t="s">
-        <v>143</v>
-      </c>
-      <c r="E32" s="6" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="33" ht="15.75" customHeight="1">
-      <c r="D33" s="6" t="s">
-        <v>145</v>
-      </c>
-      <c r="E33" s="6" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="34" ht="15.75" customHeight="1">
-      <c r="D34" s="6" t="s">
-        <v>146</v>
-      </c>
-      <c r="E34" s="6" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="35" ht="15.75" customHeight="1">
-      <c r="D35" s="6" t="s">
-        <v>147</v>
-      </c>
-      <c r="E35" s="6" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="36" ht="15.75" customHeight="1">
-      <c r="D36" s="6" t="s">
-        <v>76</v>
-      </c>
-      <c r="E36" s="6" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="37" ht="15.75" customHeight="1">
-      <c r="D37" s="6" t="s">
-        <v>149</v>
-      </c>
-      <c r="E37" s="6" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="38" ht="15.75" customHeight="1">
-      <c r="D38" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="E38" s="6" t="s">
-        <v>151</v>
+      <c r="E38" s="4" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1">
-      <c r="D39" s="6" t="s">
-        <v>152</v>
-      </c>
-      <c r="E39" s="6" t="s">
-        <v>153</v>
+      <c r="D39" s="4" t="s">
+        <v>155</v>
+      </c>
+      <c r="E39" s="4" t="s">
+        <v>157</v>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1">
-      <c r="D40" s="6" t="s">
-        <v>154</v>
-      </c>
-      <c r="E40" s="6" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="41" ht="15.75" customHeight="1"/>
-    <row r="42" ht="15.75" customHeight="1"/>
-    <row r="43" ht="15.75" customHeight="1"/>
-    <row r="44" ht="15.75" customHeight="1"/>
-    <row r="45" ht="15.75" customHeight="1"/>
-    <row r="46" ht="15.75" customHeight="1"/>
-    <row r="47" ht="15.75" customHeight="1"/>
-    <row r="48" ht="15.75" customHeight="1"/>
-    <row r="49" ht="15.75" customHeight="1"/>
+      <c r="D40" s="4" t="s">
+        <v>159</v>
+      </c>
+      <c r="E40" s="4" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="41" ht="15.75" customHeight="1">
+      <c r="D41" s="12" t="s">
+        <v>162</v>
+      </c>
+      <c r="E41" s="12" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="42" ht="15.75" customHeight="1">
+      <c r="D42" s="12" t="s">
+        <v>165</v>
+      </c>
+      <c r="E42" s="12" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="43" ht="15.75" customHeight="1">
+      <c r="D43" s="12" t="s">
+        <v>167</v>
+      </c>
+      <c r="E43" s="12" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="44" ht="15.75" customHeight="1">
+      <c r="D44" s="12" t="s">
+        <v>169</v>
+      </c>
+      <c r="E44" s="12" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="45" ht="15.75" customHeight="1">
+      <c r="D45" s="12" t="s">
+        <v>171</v>
+      </c>
+      <c r="E45" s="12" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="46" ht="15.75" customHeight="1">
+      <c r="D46" s="16"/>
+      <c r="E46" s="16"/>
+    </row>
+    <row r="47" ht="15.75" customHeight="1">
+      <c r="D47" s="16"/>
+      <c r="E47" s="16"/>
+    </row>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="D48" s="16"/>
+      <c r="E48" s="16"/>
+    </row>
+    <row r="49" ht="15.75" customHeight="1">
+      <c r="D49" s="16"/>
+      <c r="E49" s="16"/>
+    </row>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>
     <row r="52" ht="15.75" customHeight="1"/>
@@ -7278,86 +7358,86 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="4" t="s">
-        <v>12</v>
-      </c>
-    </row>
     <row r="4">
-      <c r="A4" s="6" t="s">
-        <v>19</v>
+      <c r="A4" s="4" t="s">
+        <v>6</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="7" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="6" t="s">
+    <row r="11">
+      <c r="A11" s="4" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="4" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="6" t="s">
+    <row r="15">
+      <c r="A15" s="4"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="4" t="s">
-        <v>39</v>
-      </c>
-    </row>
     <row r="17">
-      <c r="A17" s="6" t="s">
-        <v>42</v>
+      <c r="A17" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="s">
+      <c r="A18" s="4" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="4" t="s">
         <v>43</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="6" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1"/>

</xml_diff>